<commit_message>
Update event details and speaker information for SPMPQ 2026
- Revised session titles and descriptions in the program schedule to reflect accurate topics and speakers.
- Updated speaker images and added new profiles for Alexsandra Santos, Amanda Perez, Bárbara Nunes, Carolina Nanque, Clara Maia, and others to enhance the visual representation of the event.
- Removed outdated speaker data from the CSV file to streamline information management.
- Improved styling for badges and buttons in index.html for better user interaction and visual consistency.
</commit_message>
<xml_diff>
--- a/spmpq/schedule/programacao-preliminar.xlsx
+++ b/spmpq/schedule/programacao-preliminar.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
   <si>
     <t xml:space="preserve">
  II Simpósio Pernambucano Multidisciplinar de Prevenção de Quedas
@@ -331,7 +331,9 @@
 (45 min)</t>
   </si>
   <si>
-    <t xml:space="preserve">PALESTRA CIENTÍFICA                                                                                                      Fragilidade, Sarcopenia e Quedas no Hospital: O que Já Sabemos e o que Precisamos Fazer?</t>
+    <t xml:space="preserve">PALESTRA CIENTÍFICA  
+Além da capacidade funcional: autoeficácia, confiança funcional e os mecanismos invisíveis do risco de quedas em pessoas idosas     
+                                                                 </t>
   </si>
   <si>
     <t xml:space="preserve">Carolina Nanque
@@ -445,9 +447,6 @@
     <t xml:space="preserve">17h35 - 17h45 (10 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">Cecília Prado (Fisioterapeuta) - Hospital da Pessoa Idosa Recife</t>
-  </si>
-  <si>
     <t xml:space="preserve">17h45 - 17h55 (10 min) </t>
   </si>
   <si>
@@ -455,9 +454,6 @@
   </si>
   <si>
     <t xml:space="preserve">17h55 - 18h05 (10 min) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fábia Lima (Enfermeira) – Oswaldo Cruz </t>
   </si>
   <si>
     <t xml:space="preserve">18h05 - 18h10 (10 min) </t>
@@ -467,12 +463,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11.000000"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="10.000000"/>
@@ -598,7 +600,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="33">
+  <borders count="26">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -754,10 +756,10 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
         <color indexed="16"/>
@@ -767,16 +769,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
@@ -785,13 +787,13 @@
         <color indexed="16"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
@@ -802,32 +804,6 @@
       <right style="none"/>
       <top style="none"/>
       <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="none"/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal style="none"/>
     </border>
     <border>
@@ -850,17 +826,17 @@
         <color indexed="16"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="none"/>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="none"/>
       <diagonal style="none"/>
@@ -868,11 +844,22 @@
     <border>
       <left style="none"/>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="none"/>
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
@@ -886,42 +873,29 @@
       <top style="thin">
         <color auto="1"/>
       </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="none"/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left style="none"/>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
+        <color indexed="16"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="none"/>
-      <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
         <color auto="1"/>
@@ -931,344 +905,275 @@
     <border>
       <left style="none"/>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="none"/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="thin">
-        <color indexed="64"/>
+        <color indexed="16"/>
       </right>
       <top style="thin">
         <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="none"/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="thin">
-        <color indexed="16"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="thin">
-        <color indexed="16"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
       </top>
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="93">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf fontId="2" fillId="2" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="2" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="4" fillId="3" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="5" fillId="3" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf fontId="4" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="4" fillId="4" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="4" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf fontId="2" fillId="2" borderId="7" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="2" borderId="7" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="1" fillId="6" borderId="10" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="2" fillId="6" borderId="10" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="6" borderId="11" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="6" borderId="11" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="5" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="1" fillId="7" borderId="10" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="5" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="2" fillId="7" borderId="10" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="2" borderId="13" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="2" borderId="13" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="2" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="2" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="15" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="15" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="8" borderId="16" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="8" borderId="16" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="8" borderId="17" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="8" borderId="4" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="18" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="1" fillId="2" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="17" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="18" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="1" fillId="9" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="1" fillId="10" borderId="14" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="10" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="10" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="2" borderId="11" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="19" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="4" fillId="3" borderId="20" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="1" fillId="6" borderId="1" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="6" borderId="21" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="22" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="1" fillId="2" borderId="17" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="18" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="24" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="2" borderId="18" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf fontId="5" fillId="2" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="8" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="8" borderId="18" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="11" borderId="16" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="11" borderId="17" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="9" borderId="18" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf fontId="1" fillId="2" borderId="25" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="5" fillId="2" borderId="25" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="2" borderId="25" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="12" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="12" borderId="26" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="12" borderId="27" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="7" borderId="23" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="7" borderId="23" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="13" borderId="16" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="13" borderId="28" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="9" borderId="29" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="1" fillId="2" borderId="25" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="24" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="24" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="30" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="30" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf fontId="2" fillId="12" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="12" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="14" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="14" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="2" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="3" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="2" fillId="9" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="2" fillId="10" borderId="14" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="10" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="10" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="2" borderId="11" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="17" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="2" fillId="0" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="5" fillId="3" borderId="18" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="6" borderId="1" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="6" borderId="19" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="20" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="4" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="2" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="21" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="2" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="8" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="8" borderId="6" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="11" borderId="16" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="11" borderId="4" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="9" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="22" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="2" borderId="22" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="22" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="12" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="12" borderId="4" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="12" borderId="6" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="7" borderId="14" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="7" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="13" borderId="16" numFmtId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="13" borderId="4" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="9" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="22" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="21" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="2" fillId="0" borderId="21" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="2" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="3" fillId="12" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="12" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="14" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="14" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="2" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="15" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="15" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="13" borderId="16" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="6" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="6" borderId="4" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5" borderId="24" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="3" fillId="13" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="13" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="13" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="16" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="6" borderId="25" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf fontId="2" fillId="15" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf fontId="3" fillId="2" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="1" fillId="15" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="13" borderId="16" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="13" borderId="17" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="9" borderId="18" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="1" fillId="2" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="6" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="6" borderId="17" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="5" borderId="31" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="2" fillId="13" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="13" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="13" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="16" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="6" borderId="32" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="15" borderId="14" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="2" borderId="23" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf fontId="2" fillId="2" borderId="23" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperligação" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1949,13 +1854,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="1" width="12.5703125"/>
-    <col customWidth="1" min="2" max="2" style="1" width="65.28515625"/>
-    <col customWidth="1" min="3" max="3" style="2" width="26.140625"/>
-    <col customWidth="1" min="4" max="25" style="1" width="8.7109375"/>
-    <col min="26" max="16384" style="1" width="14.42578125"/>
+    <col customWidth="1" min="1" max="1" style="1" width="12.54296875"/>
+    <col customWidth="1" min="2" max="2" style="1" width="65.26953125"/>
+    <col customWidth="1" min="3" max="3" style="2" width="26.1796875"/>
+    <col customWidth="1" min="4" max="25" style="1" width="8.7265625"/>
+    <col min="26" max="16384" style="1" width="14.453125"/>
   </cols>
   <sheetData>
     <row r="1" ht="54" customHeight="1">
@@ -2378,10 +2283,10 @@
       <c r="A41" s="79" t="s">
         <v>87</v>
       </c>
-      <c r="B41" s="80" t="s">
+      <c r="B41" s="65" t="s">
         <v>88</v>
       </c>
-      <c r="C41" s="81"/>
+      <c r="C41" s="66"/>
     </row>
     <row r="42" ht="27.75" customHeight="1">
       <c r="A42" s="67"/>
@@ -2408,19 +2313,19 @@
     </row>
     <row r="45" ht="27.75" customHeight="1">
       <c r="A45" s="70"/>
-      <c r="B45" s="82" t="s">
+      <c r="B45" s="80" t="s">
         <v>93</v>
       </c>
       <c r="C45" s="71"/>
     </row>
     <row r="46" s="13" customFormat="1" ht="42" customHeight="1">
-      <c r="A46" s="83" t="s">
+      <c r="A46" s="81" t="s">
         <v>94</v>
       </c>
-      <c r="B46" s="84" t="s">
+      <c r="B46" s="82" t="s">
         <v>95</v>
       </c>
-      <c r="C46" s="85"/>
+      <c r="C46" s="83"/>
     </row>
     <row r="47" ht="27.75" customHeight="1">
       <c r="A47" s="26" t="s">
@@ -2553,33 +2458,33 @@
       <c r="Y50" s="29"/>
     </row>
     <row r="51" s="30" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A51" s="86" t="s">
+      <c r="A51" s="84" t="s">
         <v>105</v>
       </c>
-      <c r="B51" s="87" t="s">
+      <c r="B51" s="85" t="s">
         <v>106</v>
       </c>
-      <c r="C51" s="88" t="s">
+      <c r="C51" s="86" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="52" ht="42" customHeight="1">
-      <c r="A52" s="89" t="s">
+      <c r="A52" s="87" t="s">
         <v>108</v>
       </c>
       <c r="B52" s="39" t="s">
         <v>109</v>
       </c>
-      <c r="C52" s="90"/>
+      <c r="C52" s="88"/>
     </row>
     <row r="53" ht="27.75" customHeight="1">
-      <c r="A53" s="91" t="s">
+      <c r="A53" s="89" t="s">
         <v>110</v>
       </c>
-      <c r="B53" s="92" t="s">
+      <c r="B53" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="C53" s="92" t="s">
+      <c r="C53" s="20" t="s">
         <v>112</v>
       </c>
       <c r="D53" s="29"/>
@@ -2606,13 +2511,11 @@
       <c r="Y53" s="29"/>
     </row>
     <row r="54" ht="27.75" customHeight="1">
-      <c r="A54" s="91" t="s">
+      <c r="A54" s="89" t="s">
         <v>113</v>
       </c>
       <c r="B54" s="42"/>
-      <c r="C54" s="63" t="s">
-        <v>114</v>
-      </c>
+      <c r="C54" s="63"/>
       <c r="D54" s="29"/>
       <c r="E54" s="29"/>
       <c r="F54" s="29"/>
@@ -2637,12 +2540,12 @@
       <c r="Y54" s="29"/>
     </row>
     <row r="55" ht="27.75" customHeight="1">
-      <c r="A55" s="91" t="s">
+      <c r="A55" s="89" t="s">
+        <v>114</v>
+      </c>
+      <c r="B55" s="42"/>
+      <c r="C55" s="20" t="s">
         <v>115</v>
-      </c>
-      <c r="B55" s="42"/>
-      <c r="C55" s="92" t="s">
-        <v>116</v>
       </c>
       <c r="D55" s="29"/>
       <c r="E55" s="29"/>
@@ -2668,13 +2571,11 @@
       <c r="Y55" s="29"/>
     </row>
     <row r="56" ht="27.75" customHeight="1">
-      <c r="A56" s="91" t="s">
-        <v>117</v>
+      <c r="A56" s="89" t="s">
+        <v>116</v>
       </c>
       <c r="B56" s="42"/>
-      <c r="C56" s="92" t="s">
-        <v>118</v>
-      </c>
+      <c r="C56" s="20"/>
       <c r="D56" s="29"/>
       <c r="E56" s="29"/>
       <c r="F56" s="29"/>
@@ -2699,13 +2600,13 @@
       <c r="Y56" s="29"/>
     </row>
     <row r="57" ht="27.75" customHeight="1">
-      <c r="A57" s="91" t="s">
-        <v>119</v>
-      </c>
-      <c r="B57" s="93" t="s">
+      <c r="A57" s="89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B57" s="90" t="s">
         <v>39</v>
       </c>
-      <c r="C57" s="94"/>
+      <c r="C57" s="91"/>
       <c r="D57" s="29"/>
       <c r="E57" s="29"/>
       <c r="F57" s="29"/>
@@ -2730,2824 +2631,2824 @@
       <c r="Y57" s="29"/>
     </row>
     <row r="58" ht="11.25" customHeight="1">
-      <c r="B58" s="95"/>
+      <c r="B58" s="92"/>
     </row>
     <row r="59" ht="11.25" customHeight="1">
-      <c r="B59" s="95"/>
+      <c r="B59" s="92"/>
     </row>
     <row r="60" ht="11.25" customHeight="1">
-      <c r="B60" s="95"/>
+      <c r="B60" s="92"/>
     </row>
     <row r="61" ht="11.25" customHeight="1">
-      <c r="B61" s="95"/>
+      <c r="B61" s="92"/>
     </row>
     <row r="62" ht="11.25" customHeight="1">
-      <c r="B62" s="95"/>
+      <c r="B62" s="92"/>
     </row>
     <row r="63" ht="11.25" customHeight="1">
-      <c r="B63" s="95"/>
+      <c r="B63" s="92"/>
     </row>
     <row r="64" ht="11.25" customHeight="1">
-      <c r="B64" s="95"/>
+      <c r="B64" s="92"/>
     </row>
     <row r="65" ht="11.25" customHeight="1">
-      <c r="B65" s="95"/>
+      <c r="B65" s="92"/>
     </row>
     <row r="66" ht="11.25" customHeight="1">
-      <c r="B66" s="95"/>
+      <c r="B66" s="92"/>
     </row>
     <row r="67" ht="11.25" customHeight="1">
-      <c r="B67" s="95"/>
+      <c r="B67" s="92"/>
     </row>
     <row r="68" ht="11.25" customHeight="1">
-      <c r="B68" s="95"/>
+      <c r="B68" s="92"/>
     </row>
     <row r="69" ht="11.25" customHeight="1">
-      <c r="B69" s="95"/>
+      <c r="B69" s="92"/>
     </row>
     <row r="70" ht="11.25" customHeight="1">
-      <c r="B70" s="95"/>
+      <c r="B70" s="92"/>
     </row>
     <row r="71" ht="11.25" customHeight="1">
-      <c r="B71" s="95"/>
+      <c r="B71" s="92"/>
     </row>
     <row r="72" ht="11.25" customHeight="1">
-      <c r="B72" s="95"/>
+      <c r="B72" s="92"/>
     </row>
     <row r="73" ht="11.25" customHeight="1">
-      <c r="B73" s="95"/>
+      <c r="B73" s="92"/>
     </row>
     <row r="74" ht="11.25" customHeight="1">
-      <c r="B74" s="95"/>
+      <c r="B74" s="92"/>
     </row>
     <row r="75" ht="11.25" customHeight="1">
-      <c r="B75" s="95"/>
+      <c r="B75" s="92"/>
     </row>
     <row r="76" ht="11.25" customHeight="1">
-      <c r="B76" s="95"/>
+      <c r="B76" s="92"/>
     </row>
     <row r="77" ht="11.25" customHeight="1">
-      <c r="B77" s="95"/>
+      <c r="B77" s="92"/>
     </row>
     <row r="78" ht="11.25" customHeight="1">
-      <c r="B78" s="95"/>
+      <c r="B78" s="92"/>
     </row>
     <row r="79" ht="11.25" customHeight="1">
-      <c r="B79" s="95"/>
+      <c r="B79" s="92"/>
     </row>
     <row r="80" ht="11.25" customHeight="1">
-      <c r="B80" s="95"/>
+      <c r="B80" s="92"/>
     </row>
     <row r="81" ht="11.25" customHeight="1">
-      <c r="B81" s="95"/>
+      <c r="B81" s="92"/>
     </row>
     <row r="82" ht="11.25" customHeight="1">
-      <c r="B82" s="95"/>
+      <c r="B82" s="92"/>
     </row>
     <row r="83" ht="11.25" customHeight="1">
-      <c r="B83" s="95"/>
+      <c r="B83" s="92"/>
     </row>
     <row r="84" ht="11.25" customHeight="1">
-      <c r="B84" s="95"/>
+      <c r="B84" s="92"/>
     </row>
     <row r="85" ht="11.25" customHeight="1">
-      <c r="B85" s="95"/>
+      <c r="B85" s="92"/>
     </row>
     <row r="86" ht="11.25" customHeight="1">
-      <c r="B86" s="95"/>
+      <c r="B86" s="92"/>
     </row>
     <row r="87" ht="11.25" customHeight="1">
-      <c r="B87" s="95"/>
+      <c r="B87" s="92"/>
     </row>
     <row r="88" ht="11.25" customHeight="1">
-      <c r="B88" s="95"/>
+      <c r="B88" s="92"/>
     </row>
     <row r="89" ht="11.25" customHeight="1">
-      <c r="B89" s="95"/>
+      <c r="B89" s="92"/>
     </row>
     <row r="90" ht="11.25" customHeight="1">
-      <c r="B90" s="95"/>
+      <c r="B90" s="92"/>
     </row>
     <row r="91" ht="11.25" customHeight="1">
-      <c r="B91" s="95"/>
+      <c r="B91" s="92"/>
     </row>
     <row r="92" ht="11.25" customHeight="1">
-      <c r="B92" s="95"/>
+      <c r="B92" s="92"/>
     </row>
     <row r="93" ht="11.25" customHeight="1">
-      <c r="B93" s="95"/>
+      <c r="B93" s="92"/>
     </row>
     <row r="94" ht="11.25" customHeight="1">
-      <c r="B94" s="95"/>
+      <c r="B94" s="92"/>
     </row>
     <row r="95" ht="11.25" customHeight="1">
-      <c r="B95" s="95"/>
+      <c r="B95" s="92"/>
     </row>
     <row r="96" ht="11.25" customHeight="1">
-      <c r="B96" s="95"/>
+      <c r="B96" s="92"/>
     </row>
     <row r="97" ht="11.25" customHeight="1">
-      <c r="B97" s="95"/>
+      <c r="B97" s="92"/>
     </row>
     <row r="98" ht="11.25" customHeight="1">
-      <c r="B98" s="95"/>
+      <c r="B98" s="92"/>
     </row>
     <row r="99" ht="11.25" customHeight="1">
-      <c r="B99" s="95"/>
+      <c r="B99" s="92"/>
     </row>
     <row r="100" ht="11.25" customHeight="1">
-      <c r="B100" s="95"/>
+      <c r="B100" s="92"/>
     </row>
     <row r="101" ht="11.25" customHeight="1">
-      <c r="B101" s="95"/>
+      <c r="B101" s="92"/>
     </row>
     <row r="102" ht="11.25" customHeight="1">
-      <c r="B102" s="95"/>
+      <c r="B102" s="92"/>
     </row>
     <row r="103" ht="11.25" customHeight="1">
-      <c r="B103" s="95"/>
+      <c r="B103" s="92"/>
     </row>
     <row r="104" ht="11.25" customHeight="1">
-      <c r="B104" s="95"/>
+      <c r="B104" s="92"/>
     </row>
     <row r="105" ht="11.25" customHeight="1">
-      <c r="B105" s="95"/>
+      <c r="B105" s="92"/>
     </row>
     <row r="106" ht="11.25" customHeight="1">
-      <c r="B106" s="95"/>
+      <c r="B106" s="92"/>
     </row>
     <row r="107" ht="11.25" customHeight="1">
-      <c r="B107" s="95"/>
+      <c r="B107" s="92"/>
     </row>
     <row r="108" ht="11.25" customHeight="1">
-      <c r="B108" s="95"/>
+      <c r="B108" s="92"/>
     </row>
     <row r="109" ht="11.25" customHeight="1">
-      <c r="B109" s="95"/>
+      <c r="B109" s="92"/>
     </row>
     <row r="110" ht="11.25" customHeight="1">
-      <c r="B110" s="95"/>
+      <c r="B110" s="92"/>
     </row>
     <row r="111" ht="11.25" customHeight="1">
-      <c r="B111" s="95"/>
+      <c r="B111" s="92"/>
     </row>
     <row r="112" ht="11.25" customHeight="1">
-      <c r="B112" s="95"/>
+      <c r="B112" s="92"/>
     </row>
     <row r="113" ht="11.25" customHeight="1">
-      <c r="B113" s="95"/>
+      <c r="B113" s="92"/>
     </row>
     <row r="114" ht="11.25" customHeight="1">
-      <c r="B114" s="95"/>
+      <c r="B114" s="92"/>
     </row>
     <row r="115" ht="11.25" customHeight="1">
-      <c r="B115" s="95"/>
+      <c r="B115" s="92"/>
     </row>
     <row r="116" ht="11.25" customHeight="1">
-      <c r="B116" s="95"/>
+      <c r="B116" s="92"/>
     </row>
     <row r="117" ht="11.25" customHeight="1">
-      <c r="B117" s="95"/>
+      <c r="B117" s="92"/>
     </row>
     <row r="118" ht="11.25" customHeight="1">
-      <c r="B118" s="95"/>
+      <c r="B118" s="92"/>
     </row>
     <row r="119" ht="11.25" customHeight="1">
-      <c r="B119" s="95"/>
+      <c r="B119" s="92"/>
     </row>
     <row r="120" ht="11.25" customHeight="1">
-      <c r="B120" s="95"/>
+      <c r="B120" s="92"/>
     </row>
     <row r="121" ht="11.25" customHeight="1">
-      <c r="B121" s="95"/>
+      <c r="B121" s="92"/>
     </row>
     <row r="122" ht="11.25" customHeight="1">
-      <c r="B122" s="95"/>
+      <c r="B122" s="92"/>
     </row>
     <row r="123" ht="11.25" customHeight="1">
-      <c r="B123" s="95"/>
+      <c r="B123" s="92"/>
     </row>
     <row r="124" ht="11.25" customHeight="1">
-      <c r="B124" s="95"/>
+      <c r="B124" s="92"/>
     </row>
     <row r="125" ht="11.25" customHeight="1">
-      <c r="B125" s="95"/>
+      <c r="B125" s="92"/>
     </row>
     <row r="126" ht="11.25" customHeight="1">
-      <c r="B126" s="95"/>
+      <c r="B126" s="92"/>
     </row>
     <row r="127" ht="11.25" customHeight="1">
-      <c r="B127" s="95"/>
+      <c r="B127" s="92"/>
     </row>
     <row r="128" ht="11.25" customHeight="1">
-      <c r="B128" s="95"/>
+      <c r="B128" s="92"/>
     </row>
     <row r="129" ht="11.25" customHeight="1">
-      <c r="B129" s="95"/>
+      <c r="B129" s="92"/>
     </row>
     <row r="130" ht="11.25" customHeight="1">
-      <c r="B130" s="95"/>
+      <c r="B130" s="92"/>
     </row>
     <row r="131" ht="11.25" customHeight="1">
-      <c r="B131" s="95"/>
+      <c r="B131" s="92"/>
     </row>
     <row r="132" ht="11.25" customHeight="1">
-      <c r="B132" s="95"/>
+      <c r="B132" s="92"/>
     </row>
     <row r="133" ht="11.25" customHeight="1">
-      <c r="B133" s="95"/>
+      <c r="B133" s="92"/>
     </row>
     <row r="134" ht="11.25" customHeight="1">
-      <c r="B134" s="95"/>
+      <c r="B134" s="92"/>
     </row>
     <row r="135" ht="11.25" customHeight="1">
-      <c r="B135" s="95"/>
+      <c r="B135" s="92"/>
     </row>
     <row r="136" ht="11.25" customHeight="1">
-      <c r="B136" s="95"/>
+      <c r="B136" s="92"/>
     </row>
     <row r="137" ht="11.25" customHeight="1">
-      <c r="B137" s="95"/>
+      <c r="B137" s="92"/>
     </row>
     <row r="138" ht="11.25" customHeight="1">
-      <c r="B138" s="95"/>
+      <c r="B138" s="92"/>
     </row>
     <row r="139" ht="11.25" customHeight="1">
-      <c r="B139" s="95"/>
+      <c r="B139" s="92"/>
     </row>
     <row r="140" ht="11.25" customHeight="1">
-      <c r="B140" s="95"/>
+      <c r="B140" s="92"/>
     </row>
     <row r="141" ht="11.25" customHeight="1">
-      <c r="B141" s="95"/>
+      <c r="B141" s="92"/>
     </row>
     <row r="142" ht="11.25" customHeight="1">
-      <c r="B142" s="95"/>
+      <c r="B142" s="92"/>
     </row>
     <row r="143" ht="11.25" customHeight="1">
-      <c r="B143" s="95"/>
+      <c r="B143" s="92"/>
     </row>
     <row r="144" ht="11.25" customHeight="1">
-      <c r="B144" s="95"/>
+      <c r="B144" s="92"/>
     </row>
     <row r="145" ht="11.25" customHeight="1">
-      <c r="B145" s="95"/>
+      <c r="B145" s="92"/>
     </row>
     <row r="146" ht="11.25" customHeight="1">
-      <c r="B146" s="95"/>
+      <c r="B146" s="92"/>
     </row>
     <row r="147" ht="11.25" customHeight="1">
-      <c r="B147" s="95"/>
+      <c r="B147" s="92"/>
     </row>
     <row r="148" ht="11.25" customHeight="1">
-      <c r="B148" s="95"/>
+      <c r="B148" s="92"/>
     </row>
     <row r="149" ht="11.25" customHeight="1">
-      <c r="B149" s="95"/>
+      <c r="B149" s="92"/>
     </row>
     <row r="150" ht="11.25" customHeight="1">
-      <c r="B150" s="95"/>
+      <c r="B150" s="92"/>
     </row>
     <row r="151" ht="11.25" customHeight="1">
-      <c r="B151" s="95"/>
+      <c r="B151" s="92"/>
     </row>
     <row r="152" ht="11.25" customHeight="1">
-      <c r="B152" s="95"/>
+      <c r="B152" s="92"/>
     </row>
     <row r="153" ht="11.25" customHeight="1">
-      <c r="B153" s="95"/>
+      <c r="B153" s="92"/>
     </row>
     <row r="154" ht="11.25" customHeight="1">
-      <c r="B154" s="95"/>
+      <c r="B154" s="92"/>
     </row>
     <row r="155" ht="11.25" customHeight="1">
-      <c r="B155" s="95"/>
+      <c r="B155" s="92"/>
     </row>
     <row r="156" ht="11.25" customHeight="1">
-      <c r="B156" s="95"/>
+      <c r="B156" s="92"/>
     </row>
     <row r="157" ht="11.25" customHeight="1">
-      <c r="B157" s="95"/>
+      <c r="B157" s="92"/>
     </row>
     <row r="158" ht="11.25" customHeight="1">
-      <c r="B158" s="95"/>
+      <c r="B158" s="92"/>
     </row>
     <row r="159" ht="11.25" customHeight="1">
-      <c r="B159" s="95"/>
+      <c r="B159" s="92"/>
     </row>
     <row r="160" ht="11.25" customHeight="1">
-      <c r="B160" s="95"/>
+      <c r="B160" s="92"/>
     </row>
     <row r="161" ht="11.25" customHeight="1">
-      <c r="B161" s="95"/>
+      <c r="B161" s="92"/>
     </row>
     <row r="162" ht="11.25" customHeight="1">
-      <c r="B162" s="95"/>
+      <c r="B162" s="92"/>
     </row>
     <row r="163" ht="11.25" customHeight="1">
-      <c r="B163" s="95"/>
+      <c r="B163" s="92"/>
     </row>
     <row r="164" ht="11.25" customHeight="1">
-      <c r="B164" s="95"/>
+      <c r="B164" s="92"/>
     </row>
     <row r="165" ht="11.25" customHeight="1">
-      <c r="B165" s="95"/>
+      <c r="B165" s="92"/>
     </row>
     <row r="166" ht="11.25" customHeight="1">
-      <c r="B166" s="95"/>
+      <c r="B166" s="92"/>
     </row>
     <row r="167" ht="11.25" customHeight="1">
-      <c r="B167" s="95"/>
+      <c r="B167" s="92"/>
     </row>
     <row r="168" ht="11.25" customHeight="1">
-      <c r="B168" s="95"/>
+      <c r="B168" s="92"/>
     </row>
     <row r="169" ht="11.25" customHeight="1">
-      <c r="B169" s="95"/>
+      <c r="B169" s="92"/>
     </row>
     <row r="170" ht="11.25" customHeight="1">
-      <c r="B170" s="95"/>
+      <c r="B170" s="92"/>
     </row>
     <row r="171" ht="11.25" customHeight="1">
-      <c r="B171" s="95"/>
+      <c r="B171" s="92"/>
     </row>
     <row r="172" ht="11.25" customHeight="1">
-      <c r="B172" s="95"/>
+      <c r="B172" s="92"/>
     </row>
     <row r="173" ht="11.25" customHeight="1">
-      <c r="B173" s="95"/>
+      <c r="B173" s="92"/>
     </row>
     <row r="174" ht="11.25" customHeight="1">
-      <c r="B174" s="95"/>
+      <c r="B174" s="92"/>
     </row>
     <row r="175" ht="11.25" customHeight="1">
-      <c r="B175" s="95"/>
+      <c r="B175" s="92"/>
     </row>
     <row r="176" ht="11.25" customHeight="1">
-      <c r="B176" s="95"/>
+      <c r="B176" s="92"/>
     </row>
     <row r="177" ht="11.25" customHeight="1">
-      <c r="B177" s="95"/>
+      <c r="B177" s="92"/>
     </row>
     <row r="178" ht="11.25" customHeight="1">
-      <c r="B178" s="95"/>
+      <c r="B178" s="92"/>
     </row>
     <row r="179" ht="11.25" customHeight="1">
-      <c r="B179" s="95"/>
+      <c r="B179" s="92"/>
     </row>
     <row r="180" ht="11.25" customHeight="1">
-      <c r="B180" s="95"/>
+      <c r="B180" s="92"/>
     </row>
     <row r="181" ht="11.25" customHeight="1">
-      <c r="B181" s="95"/>
+      <c r="B181" s="92"/>
     </row>
     <row r="182" ht="11.25" customHeight="1">
-      <c r="B182" s="95"/>
+      <c r="B182" s="92"/>
     </row>
     <row r="183" ht="11.25" customHeight="1">
-      <c r="B183" s="95"/>
+      <c r="B183" s="92"/>
     </row>
     <row r="184" ht="11.25" customHeight="1">
-      <c r="B184" s="95"/>
+      <c r="B184" s="92"/>
     </row>
     <row r="185" ht="11.25" customHeight="1">
-      <c r="B185" s="95"/>
+      <c r="B185" s="92"/>
     </row>
     <row r="186" ht="11.25" customHeight="1">
-      <c r="B186" s="95"/>
+      <c r="B186" s="92"/>
     </row>
     <row r="187" ht="11.25" customHeight="1">
-      <c r="B187" s="95"/>
+      <c r="B187" s="92"/>
     </row>
     <row r="188" ht="11.25" customHeight="1">
-      <c r="B188" s="95"/>
+      <c r="B188" s="92"/>
     </row>
     <row r="189" ht="11.25" customHeight="1">
-      <c r="B189" s="95"/>
+      <c r="B189" s="92"/>
     </row>
     <row r="190" ht="11.25" customHeight="1">
-      <c r="B190" s="95"/>
+      <c r="B190" s="92"/>
     </row>
     <row r="191" ht="11.25" customHeight="1">
-      <c r="B191" s="95"/>
+      <c r="B191" s="92"/>
     </row>
     <row r="192" ht="11.25" customHeight="1">
-      <c r="B192" s="95"/>
+      <c r="B192" s="92"/>
     </row>
     <row r="193" ht="11.25" customHeight="1">
-      <c r="B193" s="95"/>
+      <c r="B193" s="92"/>
     </row>
     <row r="194" ht="11.25" customHeight="1">
-      <c r="B194" s="95"/>
+      <c r="B194" s="92"/>
     </row>
     <row r="195" ht="11.25" customHeight="1">
-      <c r="B195" s="95"/>
+      <c r="B195" s="92"/>
     </row>
     <row r="196" ht="11.25" customHeight="1">
-      <c r="B196" s="95"/>
+      <c r="B196" s="92"/>
     </row>
     <row r="197" ht="11.25" customHeight="1">
-      <c r="B197" s="95"/>
+      <c r="B197" s="92"/>
     </row>
     <row r="198" ht="11.25" customHeight="1">
-      <c r="B198" s="95"/>
+      <c r="B198" s="92"/>
     </row>
     <row r="199" ht="11.25" customHeight="1">
-      <c r="B199" s="95"/>
+      <c r="B199" s="92"/>
     </row>
     <row r="200" ht="11.25" customHeight="1">
-      <c r="B200" s="95"/>
+      <c r="B200" s="92"/>
     </row>
     <row r="201" ht="11.25" customHeight="1">
-      <c r="B201" s="95"/>
+      <c r="B201" s="92"/>
     </row>
     <row r="202" ht="11.25" customHeight="1">
-      <c r="B202" s="95"/>
+      <c r="B202" s="92"/>
     </row>
     <row r="203" ht="11.25" customHeight="1">
-      <c r="B203" s="95"/>
+      <c r="B203" s="92"/>
     </row>
     <row r="204" ht="11.25" customHeight="1">
-      <c r="B204" s="95"/>
+      <c r="B204" s="92"/>
     </row>
     <row r="205" ht="11.25" customHeight="1">
-      <c r="B205" s="95"/>
+      <c r="B205" s="92"/>
     </row>
     <row r="206" ht="11.25" customHeight="1">
-      <c r="B206" s="95"/>
+      <c r="B206" s="92"/>
     </row>
     <row r="207" ht="11.25" customHeight="1">
-      <c r="B207" s="95"/>
+      <c r="B207" s="92"/>
     </row>
     <row r="208" ht="11.25" customHeight="1">
-      <c r="B208" s="95"/>
+      <c r="B208" s="92"/>
     </row>
     <row r="209" ht="11.25" customHeight="1">
-      <c r="B209" s="95"/>
+      <c r="B209" s="92"/>
     </row>
     <row r="210" ht="11.25" customHeight="1">
-      <c r="B210" s="95"/>
+      <c r="B210" s="92"/>
     </row>
     <row r="211" ht="11.25" customHeight="1">
-      <c r="B211" s="95"/>
+      <c r="B211" s="92"/>
     </row>
     <row r="212" ht="11.25" customHeight="1">
-      <c r="B212" s="95"/>
+      <c r="B212" s="92"/>
     </row>
     <row r="213" ht="11.25" customHeight="1">
-      <c r="B213" s="95"/>
+      <c r="B213" s="92"/>
     </row>
     <row r="214" ht="11.25" customHeight="1">
-      <c r="B214" s="95"/>
+      <c r="B214" s="92"/>
     </row>
     <row r="215" ht="11.25" customHeight="1">
-      <c r="B215" s="95"/>
+      <c r="B215" s="92"/>
     </row>
     <row r="216" ht="11.25" customHeight="1">
-      <c r="B216" s="95"/>
+      <c r="B216" s="92"/>
     </row>
     <row r="217" ht="11.25" customHeight="1">
-      <c r="B217" s="95"/>
+      <c r="B217" s="92"/>
     </row>
     <row r="218" ht="11.25" customHeight="1">
-      <c r="B218" s="95"/>
+      <c r="B218" s="92"/>
     </row>
     <row r="219" ht="11.25" customHeight="1">
-      <c r="B219" s="95"/>
+      <c r="B219" s="92"/>
     </row>
     <row r="220" ht="11.25" customHeight="1">
-      <c r="B220" s="95"/>
+      <c r="B220" s="92"/>
     </row>
     <row r="221" ht="11.25" customHeight="1">
-      <c r="B221" s="95"/>
+      <c r="B221" s="92"/>
     </row>
     <row r="222" ht="11.25" customHeight="1">
-      <c r="B222" s="95"/>
+      <c r="B222" s="92"/>
     </row>
     <row r="223" ht="11.25" customHeight="1">
-      <c r="B223" s="95"/>
+      <c r="B223" s="92"/>
     </row>
     <row r="224" ht="11.25" customHeight="1">
-      <c r="B224" s="95"/>
+      <c r="B224" s="92"/>
     </row>
     <row r="225" ht="11.25" customHeight="1">
-      <c r="B225" s="95"/>
+      <c r="B225" s="92"/>
     </row>
     <row r="226" ht="11.25" customHeight="1">
-      <c r="B226" s="95"/>
+      <c r="B226" s="92"/>
     </row>
     <row r="227" ht="11.25" customHeight="1">
-      <c r="B227" s="95"/>
+      <c r="B227" s="92"/>
     </row>
     <row r="228" ht="11.25" customHeight="1">
-      <c r="B228" s="95"/>
+      <c r="B228" s="92"/>
     </row>
     <row r="229" ht="11.25" customHeight="1">
-      <c r="B229" s="95"/>
+      <c r="B229" s="92"/>
     </row>
     <row r="230" ht="11.25" customHeight="1">
-      <c r="B230" s="95"/>
+      <c r="B230" s="92"/>
     </row>
     <row r="231" ht="11.25" customHeight="1">
-      <c r="B231" s="95"/>
+      <c r="B231" s="92"/>
     </row>
     <row r="232" ht="11.25" customHeight="1">
-      <c r="B232" s="95"/>
+      <c r="B232" s="92"/>
     </row>
     <row r="233" ht="11.25" customHeight="1">
-      <c r="B233" s="95"/>
+      <c r="B233" s="92"/>
     </row>
     <row r="234" ht="11.25" customHeight="1">
-      <c r="B234" s="95"/>
+      <c r="B234" s="92"/>
     </row>
     <row r="235" ht="11.25" customHeight="1">
-      <c r="B235" s="95"/>
+      <c r="B235" s="92"/>
     </row>
     <row r="236" ht="11.25" customHeight="1">
-      <c r="B236" s="95"/>
+      <c r="B236" s="92"/>
     </row>
     <row r="237" ht="11.25" customHeight="1">
-      <c r="B237" s="95"/>
+      <c r="B237" s="92"/>
     </row>
     <row r="238" ht="11.25" customHeight="1">
-      <c r="B238" s="95"/>
+      <c r="B238" s="92"/>
     </row>
     <row r="239" ht="11.25" customHeight="1">
-      <c r="B239" s="95"/>
+      <c r="B239" s="92"/>
     </row>
     <row r="240" ht="11.25" customHeight="1">
-      <c r="B240" s="95"/>
+      <c r="B240" s="92"/>
     </row>
     <row r="241" ht="11.25" customHeight="1">
-      <c r="B241" s="95"/>
+      <c r="B241" s="92"/>
     </row>
     <row r="242" ht="11.25" customHeight="1">
-      <c r="B242" s="95"/>
+      <c r="B242" s="92"/>
     </row>
     <row r="243" ht="11.25" customHeight="1">
-      <c r="B243" s="95"/>
+      <c r="B243" s="92"/>
     </row>
     <row r="244" ht="11.25" customHeight="1">
-      <c r="B244" s="95"/>
+      <c r="B244" s="92"/>
     </row>
     <row r="245" ht="11.25" customHeight="1">
-      <c r="B245" s="95"/>
+      <c r="B245" s="92"/>
     </row>
     <row r="246" ht="11.25" customHeight="1">
-      <c r="B246" s="95"/>
+      <c r="B246" s="92"/>
     </row>
     <row r="247" ht="11.25" customHeight="1">
-      <c r="B247" s="95"/>
+      <c r="B247" s="92"/>
     </row>
     <row r="248" ht="11.25" customHeight="1">
-      <c r="B248" s="95"/>
+      <c r="B248" s="92"/>
     </row>
     <row r="249" ht="11.25" customHeight="1">
-      <c r="B249" s="95"/>
+      <c r="B249" s="92"/>
     </row>
     <row r="250" ht="11.25" customHeight="1">
-      <c r="B250" s="95"/>
+      <c r="B250" s="92"/>
     </row>
     <row r="251" ht="11.25" customHeight="1">
-      <c r="B251" s="95"/>
+      <c r="B251" s="92"/>
     </row>
     <row r="252" ht="11.25" customHeight="1">
-      <c r="B252" s="95"/>
+      <c r="B252" s="92"/>
     </row>
     <row r="253" ht="11.25" customHeight="1">
-      <c r="B253" s="95"/>
+      <c r="B253" s="92"/>
     </row>
     <row r="254" ht="11.25" customHeight="1">
-      <c r="B254" s="95"/>
+      <c r="B254" s="92"/>
     </row>
     <row r="255" ht="11.25" customHeight="1">
-      <c r="B255" s="95"/>
+      <c r="B255" s="92"/>
     </row>
     <row r="256" ht="11.25" customHeight="1">
-      <c r="B256" s="95"/>
+      <c r="B256" s="92"/>
     </row>
     <row r="257" ht="11.25" customHeight="1">
-      <c r="B257" s="95"/>
+      <c r="B257" s="92"/>
     </row>
     <row r="258" ht="11.25" customHeight="1">
-      <c r="B258" s="95"/>
+      <c r="B258" s="92"/>
     </row>
     <row r="259" ht="11.25" customHeight="1">
-      <c r="B259" s="95"/>
+      <c r="B259" s="92"/>
     </row>
     <row r="260" ht="11.25" customHeight="1">
-      <c r="B260" s="95"/>
+      <c r="B260" s="92"/>
     </row>
     <row r="261" ht="11.25" customHeight="1">
-      <c r="B261" s="95"/>
+      <c r="B261" s="92"/>
     </row>
     <row r="262" ht="11.25" customHeight="1">
-      <c r="B262" s="95"/>
+      <c r="B262" s="92"/>
     </row>
     <row r="263" ht="11.25" customHeight="1">
-      <c r="B263" s="95"/>
+      <c r="B263" s="92"/>
     </row>
     <row r="264" ht="11.25" customHeight="1">
-      <c r="B264" s="95"/>
+      <c r="B264" s="92"/>
     </row>
     <row r="265" ht="11.25" customHeight="1">
-      <c r="B265" s="95"/>
+      <c r="B265" s="92"/>
     </row>
     <row r="266" ht="11.25" customHeight="1">
-      <c r="B266" s="95"/>
+      <c r="B266" s="92"/>
     </row>
     <row r="267" ht="11.25" customHeight="1">
-      <c r="B267" s="95"/>
+      <c r="B267" s="92"/>
     </row>
     <row r="268" ht="11.25" customHeight="1">
-      <c r="B268" s="95"/>
+      <c r="B268" s="92"/>
     </row>
     <row r="269" ht="11.25" customHeight="1">
-      <c r="B269" s="95"/>
+      <c r="B269" s="92"/>
     </row>
     <row r="270" ht="11.25" customHeight="1">
-      <c r="B270" s="95"/>
+      <c r="B270" s="92"/>
     </row>
     <row r="271" ht="11.25" customHeight="1">
-      <c r="B271" s="95"/>
+      <c r="B271" s="92"/>
     </row>
     <row r="272" ht="11.25" customHeight="1">
-      <c r="B272" s="95"/>
+      <c r="B272" s="92"/>
     </row>
     <row r="273" ht="11.25" customHeight="1">
-      <c r="B273" s="95"/>
+      <c r="B273" s="92"/>
     </row>
     <row r="274" ht="11.25" customHeight="1">
-      <c r="B274" s="95"/>
+      <c r="B274" s="92"/>
     </row>
     <row r="275" ht="11.25" customHeight="1">
-      <c r="B275" s="95"/>
+      <c r="B275" s="92"/>
     </row>
     <row r="276" ht="11.25" customHeight="1">
-      <c r="B276" s="95"/>
+      <c r="B276" s="92"/>
     </row>
     <row r="277" ht="11.25" customHeight="1">
-      <c r="B277" s="95"/>
+      <c r="B277" s="92"/>
     </row>
     <row r="278" ht="11.25" customHeight="1">
-      <c r="B278" s="95"/>
+      <c r="B278" s="92"/>
     </row>
     <row r="279" ht="11.25" customHeight="1">
-      <c r="B279" s="95"/>
+      <c r="B279" s="92"/>
     </row>
     <row r="280" ht="11.25" customHeight="1">
-      <c r="B280" s="95"/>
+      <c r="B280" s="92"/>
     </row>
     <row r="281" ht="11.25" customHeight="1">
-      <c r="B281" s="95"/>
+      <c r="B281" s="92"/>
     </row>
     <row r="282" ht="11.25" customHeight="1">
-      <c r="B282" s="95"/>
+      <c r="B282" s="92"/>
     </row>
     <row r="283" ht="11.25" customHeight="1">
-      <c r="B283" s="95"/>
+      <c r="B283" s="92"/>
     </row>
     <row r="284" ht="11.25" customHeight="1">
-      <c r="B284" s="95"/>
+      <c r="B284" s="92"/>
     </row>
     <row r="285" ht="11.25" customHeight="1">
-      <c r="B285" s="95"/>
+      <c r="B285" s="92"/>
     </row>
     <row r="286" ht="11.25" customHeight="1">
-      <c r="B286" s="95"/>
+      <c r="B286" s="92"/>
     </row>
     <row r="287" ht="11.25" customHeight="1">
-      <c r="B287" s="95"/>
+      <c r="B287" s="92"/>
     </row>
     <row r="288" ht="11.25" customHeight="1">
-      <c r="B288" s="95"/>
+      <c r="B288" s="92"/>
     </row>
     <row r="289" ht="11.25" customHeight="1">
-      <c r="B289" s="95"/>
+      <c r="B289" s="92"/>
     </row>
     <row r="290" ht="11.25" customHeight="1">
-      <c r="B290" s="95"/>
+      <c r="B290" s="92"/>
     </row>
     <row r="291" ht="11.25" customHeight="1">
-      <c r="B291" s="95"/>
+      <c r="B291" s="92"/>
     </row>
     <row r="292" ht="11.25" customHeight="1">
-      <c r="B292" s="95"/>
+      <c r="B292" s="92"/>
     </row>
     <row r="293" ht="11.25" customHeight="1">
-      <c r="B293" s="95"/>
+      <c r="B293" s="92"/>
     </row>
     <row r="294" ht="11.25" customHeight="1">
-      <c r="B294" s="95"/>
+      <c r="B294" s="92"/>
     </row>
     <row r="295" ht="11.25" customHeight="1">
-      <c r="B295" s="95"/>
+      <c r="B295" s="92"/>
     </row>
     <row r="296" ht="11.25" customHeight="1">
-      <c r="B296" s="95"/>
+      <c r="B296" s="92"/>
     </row>
     <row r="297" ht="11.25" customHeight="1">
-      <c r="B297" s="95"/>
+      <c r="B297" s="92"/>
     </row>
     <row r="298" ht="11.25" customHeight="1">
-      <c r="B298" s="95"/>
+      <c r="B298" s="92"/>
     </row>
     <row r="299" ht="11.25" customHeight="1">
-      <c r="B299" s="95"/>
+      <c r="B299" s="92"/>
     </row>
     <row r="300" ht="11.25" customHeight="1">
-      <c r="B300" s="95"/>
+      <c r="B300" s="92"/>
     </row>
     <row r="301" ht="11.25" customHeight="1">
-      <c r="B301" s="95"/>
+      <c r="B301" s="92"/>
     </row>
     <row r="302" ht="11.25" customHeight="1">
-      <c r="B302" s="95"/>
+      <c r="B302" s="92"/>
     </row>
     <row r="303" ht="11.25" customHeight="1">
-      <c r="B303" s="95"/>
+      <c r="B303" s="92"/>
     </row>
     <row r="304" ht="11.25" customHeight="1">
-      <c r="B304" s="95"/>
+      <c r="B304" s="92"/>
     </row>
     <row r="305" ht="11.25" customHeight="1">
-      <c r="B305" s="95"/>
+      <c r="B305" s="92"/>
     </row>
     <row r="306" ht="11.25" customHeight="1">
-      <c r="B306" s="95"/>
+      <c r="B306" s="92"/>
     </row>
     <row r="307" ht="11.25" customHeight="1">
-      <c r="B307" s="95"/>
+      <c r="B307" s="92"/>
     </row>
     <row r="308" ht="11.25" customHeight="1">
-      <c r="B308" s="95"/>
+      <c r="B308" s="92"/>
     </row>
     <row r="309" ht="11.25" customHeight="1">
-      <c r="B309" s="95"/>
+      <c r="B309" s="92"/>
     </row>
     <row r="310" ht="11.25" customHeight="1">
-      <c r="B310" s="95"/>
+      <c r="B310" s="92"/>
     </row>
     <row r="311" ht="11.25" customHeight="1">
-      <c r="B311" s="95"/>
+      <c r="B311" s="92"/>
     </row>
     <row r="312" ht="11.25" customHeight="1">
-      <c r="B312" s="95"/>
+      <c r="B312" s="92"/>
     </row>
     <row r="313" ht="11.25" customHeight="1">
-      <c r="B313" s="95"/>
+      <c r="B313" s="92"/>
     </row>
     <row r="314" ht="11.25" customHeight="1">
-      <c r="B314" s="95"/>
+      <c r="B314" s="92"/>
     </row>
     <row r="315" ht="11.25" customHeight="1">
-      <c r="B315" s="95"/>
+      <c r="B315" s="92"/>
     </row>
     <row r="316" ht="11.25" customHeight="1">
-      <c r="B316" s="95"/>
+      <c r="B316" s="92"/>
     </row>
     <row r="317" ht="11.25" customHeight="1">
-      <c r="B317" s="95"/>
+      <c r="B317" s="92"/>
     </row>
     <row r="318" ht="11.25" customHeight="1">
-      <c r="B318" s="95"/>
+      <c r="B318" s="92"/>
     </row>
     <row r="319" ht="11.25" customHeight="1">
-      <c r="B319" s="95"/>
+      <c r="B319" s="92"/>
     </row>
     <row r="320" ht="11.25" customHeight="1">
-      <c r="B320" s="95"/>
+      <c r="B320" s="92"/>
     </row>
     <row r="321" ht="11.25" customHeight="1">
-      <c r="B321" s="95"/>
+      <c r="B321" s="92"/>
     </row>
     <row r="322" ht="11.25" customHeight="1">
-      <c r="B322" s="95"/>
+      <c r="B322" s="92"/>
     </row>
     <row r="323" ht="11.25" customHeight="1">
-      <c r="B323" s="95"/>
+      <c r="B323" s="92"/>
     </row>
     <row r="324" ht="11.25" customHeight="1">
-      <c r="B324" s="95"/>
+      <c r="B324" s="92"/>
     </row>
     <row r="325" ht="11.25" customHeight="1">
-      <c r="B325" s="95"/>
+      <c r="B325" s="92"/>
     </row>
     <row r="326" ht="11.25" customHeight="1">
-      <c r="B326" s="95"/>
+      <c r="B326" s="92"/>
     </row>
     <row r="327" ht="11.25" customHeight="1">
-      <c r="B327" s="95"/>
+      <c r="B327" s="92"/>
     </row>
     <row r="328" ht="11.25" customHeight="1">
-      <c r="B328" s="95"/>
+      <c r="B328" s="92"/>
     </row>
     <row r="329" ht="11.25" customHeight="1">
-      <c r="B329" s="95"/>
+      <c r="B329" s="92"/>
     </row>
     <row r="330" ht="11.25" customHeight="1">
-      <c r="B330" s="95"/>
+      <c r="B330" s="92"/>
     </row>
     <row r="331" ht="11.25" customHeight="1">
-      <c r="B331" s="95"/>
+      <c r="B331" s="92"/>
     </row>
     <row r="332" ht="11.25" customHeight="1">
-      <c r="B332" s="95"/>
+      <c r="B332" s="92"/>
     </row>
     <row r="333" ht="11.25" customHeight="1">
-      <c r="B333" s="95"/>
+      <c r="B333" s="92"/>
     </row>
     <row r="334" ht="11.25" customHeight="1">
-      <c r="B334" s="95"/>
+      <c r="B334" s="92"/>
     </row>
     <row r="335" ht="11.25" customHeight="1">
-      <c r="B335" s="95"/>
+      <c r="B335" s="92"/>
     </row>
     <row r="336" ht="11.25" customHeight="1">
-      <c r="B336" s="95"/>
+      <c r="B336" s="92"/>
     </row>
     <row r="337" ht="11.25" customHeight="1">
-      <c r="B337" s="95"/>
+      <c r="B337" s="92"/>
     </row>
     <row r="338" ht="11.25" customHeight="1">
-      <c r="B338" s="95"/>
+      <c r="B338" s="92"/>
     </row>
     <row r="339" ht="11.25" customHeight="1">
-      <c r="B339" s="95"/>
+      <c r="B339" s="92"/>
     </row>
     <row r="340" ht="11.25" customHeight="1">
-      <c r="B340" s="95"/>
+      <c r="B340" s="92"/>
     </row>
     <row r="341" ht="11.25" customHeight="1">
-      <c r="B341" s="95"/>
+      <c r="B341" s="92"/>
     </row>
     <row r="342" ht="11.25" customHeight="1">
-      <c r="B342" s="95"/>
+      <c r="B342" s="92"/>
     </row>
     <row r="343" ht="11.25" customHeight="1">
-      <c r="B343" s="95"/>
+      <c r="B343" s="92"/>
     </row>
     <row r="344" ht="11.25" customHeight="1">
-      <c r="B344" s="95"/>
+      <c r="B344" s="92"/>
     </row>
     <row r="345" ht="11.25" customHeight="1">
-      <c r="B345" s="95"/>
+      <c r="B345" s="92"/>
     </row>
     <row r="346" ht="11.25" customHeight="1">
-      <c r="B346" s="95"/>
+      <c r="B346" s="92"/>
     </row>
     <row r="347" ht="11.25" customHeight="1">
-      <c r="B347" s="95"/>
+      <c r="B347" s="92"/>
     </row>
     <row r="348" ht="11.25" customHeight="1">
-      <c r="B348" s="95"/>
+      <c r="B348" s="92"/>
     </row>
     <row r="349" ht="11.25" customHeight="1">
-      <c r="B349" s="95"/>
+      <c r="B349" s="92"/>
     </row>
     <row r="350" ht="11.25" customHeight="1">
-      <c r="B350" s="95"/>
+      <c r="B350" s="92"/>
     </row>
     <row r="351" ht="11.25" customHeight="1">
-      <c r="B351" s="95"/>
+      <c r="B351" s="92"/>
     </row>
     <row r="352" ht="11.25" customHeight="1">
-      <c r="B352" s="95"/>
+      <c r="B352" s="92"/>
     </row>
     <row r="353" ht="11.25" customHeight="1">
-      <c r="B353" s="95"/>
+      <c r="B353" s="92"/>
     </row>
     <row r="354" ht="11.25" customHeight="1">
-      <c r="B354" s="95"/>
+      <c r="B354" s="92"/>
     </row>
     <row r="355" ht="11.25" customHeight="1">
-      <c r="B355" s="95"/>
+      <c r="B355" s="92"/>
     </row>
     <row r="356" ht="11.25" customHeight="1">
-      <c r="B356" s="95"/>
+      <c r="B356" s="92"/>
     </row>
     <row r="357" ht="11.25" customHeight="1">
-      <c r="B357" s="95"/>
+      <c r="B357" s="92"/>
     </row>
     <row r="358" ht="11.25" customHeight="1">
-      <c r="B358" s="95"/>
+      <c r="B358" s="92"/>
     </row>
     <row r="359" ht="11.25" customHeight="1">
-      <c r="B359" s="95"/>
+      <c r="B359" s="92"/>
     </row>
     <row r="360" ht="11.25" customHeight="1">
-      <c r="B360" s="95"/>
+      <c r="B360" s="92"/>
     </row>
     <row r="361" ht="11.25" customHeight="1">
-      <c r="B361" s="95"/>
+      <c r="B361" s="92"/>
     </row>
     <row r="362" ht="11.25" customHeight="1">
-      <c r="B362" s="95"/>
+      <c r="B362" s="92"/>
     </row>
     <row r="363" ht="11.25" customHeight="1">
-      <c r="B363" s="95"/>
+      <c r="B363" s="92"/>
     </row>
     <row r="364" ht="11.25" customHeight="1">
-      <c r="B364" s="95"/>
+      <c r="B364" s="92"/>
     </row>
     <row r="365" ht="11.25" customHeight="1">
-      <c r="B365" s="95"/>
+      <c r="B365" s="92"/>
     </row>
     <row r="366" ht="11.25" customHeight="1">
-      <c r="B366" s="95"/>
+      <c r="B366" s="92"/>
     </row>
     <row r="367" ht="11.25" customHeight="1">
-      <c r="B367" s="95"/>
+      <c r="B367" s="92"/>
     </row>
     <row r="368" ht="11.25" customHeight="1">
-      <c r="B368" s="95"/>
+      <c r="B368" s="92"/>
     </row>
     <row r="369" ht="11.25" customHeight="1">
-      <c r="B369" s="95"/>
+      <c r="B369" s="92"/>
     </row>
     <row r="370" ht="11.25" customHeight="1">
-      <c r="B370" s="95"/>
+      <c r="B370" s="92"/>
     </row>
     <row r="371" ht="11.25" customHeight="1">
-      <c r="B371" s="95"/>
+      <c r="B371" s="92"/>
     </row>
     <row r="372" ht="11.25" customHeight="1">
-      <c r="B372" s="95"/>
+      <c r="B372" s="92"/>
     </row>
     <row r="373" ht="11.25" customHeight="1">
-      <c r="B373" s="95"/>
+      <c r="B373" s="92"/>
     </row>
     <row r="374" ht="11.25" customHeight="1">
-      <c r="B374" s="95"/>
+      <c r="B374" s="92"/>
     </row>
     <row r="375" ht="11.25" customHeight="1">
-      <c r="B375" s="95"/>
+      <c r="B375" s="92"/>
     </row>
     <row r="376" ht="11.25" customHeight="1">
-      <c r="B376" s="95"/>
+      <c r="B376" s="92"/>
     </row>
     <row r="377" ht="11.25" customHeight="1">
-      <c r="B377" s="95"/>
+      <c r="B377" s="92"/>
     </row>
     <row r="378" ht="11.25" customHeight="1">
-      <c r="B378" s="95"/>
+      <c r="B378" s="92"/>
     </row>
     <row r="379" ht="11.25" customHeight="1">
-      <c r="B379" s="95"/>
+      <c r="B379" s="92"/>
     </row>
     <row r="380" ht="11.25" customHeight="1">
-      <c r="B380" s="95"/>
+      <c r="B380" s="92"/>
     </row>
     <row r="381" ht="11.25" customHeight="1">
-      <c r="B381" s="95"/>
+      <c r="B381" s="92"/>
     </row>
     <row r="382" ht="11.25" customHeight="1">
-      <c r="B382" s="95"/>
+      <c r="B382" s="92"/>
     </row>
     <row r="383" ht="11.25" customHeight="1">
-      <c r="B383" s="95"/>
+      <c r="B383" s="92"/>
     </row>
     <row r="384" ht="11.25" customHeight="1">
-      <c r="B384" s="95"/>
+      <c r="B384" s="92"/>
     </row>
     <row r="385" ht="11.25" customHeight="1">
-      <c r="B385" s="95"/>
+      <c r="B385" s="92"/>
     </row>
     <row r="386" ht="11.25" customHeight="1">
-      <c r="B386" s="95"/>
+      <c r="B386" s="92"/>
     </row>
     <row r="387" ht="11.25" customHeight="1">
-      <c r="B387" s="95"/>
+      <c r="B387" s="92"/>
     </row>
     <row r="388" ht="11.25" customHeight="1">
-      <c r="B388" s="95"/>
+      <c r="B388" s="92"/>
     </row>
     <row r="389" ht="11.25" customHeight="1">
-      <c r="B389" s="95"/>
+      <c r="B389" s="92"/>
     </row>
     <row r="390" ht="11.25" customHeight="1">
-      <c r="B390" s="95"/>
+      <c r="B390" s="92"/>
     </row>
     <row r="391" ht="11.25" customHeight="1">
-      <c r="B391" s="95"/>
+      <c r="B391" s="92"/>
     </row>
     <row r="392" ht="11.25" customHeight="1">
-      <c r="B392" s="95"/>
+      <c r="B392" s="92"/>
     </row>
     <row r="393" ht="11.25" customHeight="1">
-      <c r="B393" s="95"/>
+      <c r="B393" s="92"/>
     </row>
     <row r="394" ht="11.25" customHeight="1">
-      <c r="B394" s="95"/>
+      <c r="B394" s="92"/>
     </row>
     <row r="395" ht="11.25" customHeight="1">
-      <c r="B395" s="95"/>
+      <c r="B395" s="92"/>
     </row>
     <row r="396" ht="11.25" customHeight="1">
-      <c r="B396" s="95"/>
+      <c r="B396" s="92"/>
     </row>
     <row r="397" ht="11.25" customHeight="1">
-      <c r="B397" s="95"/>
+      <c r="B397" s="92"/>
     </row>
     <row r="398" ht="11.25" customHeight="1">
-      <c r="B398" s="95"/>
+      <c r="B398" s="92"/>
     </row>
     <row r="399" ht="11.25" customHeight="1">
-      <c r="B399" s="95"/>
+      <c r="B399" s="92"/>
     </row>
     <row r="400" ht="11.25" customHeight="1">
-      <c r="B400" s="95"/>
+      <c r="B400" s="92"/>
     </row>
     <row r="401" ht="11.25" customHeight="1">
-      <c r="B401" s="95"/>
+      <c r="B401" s="92"/>
     </row>
     <row r="402" ht="11.25" customHeight="1">
-      <c r="B402" s="95"/>
+      <c r="B402" s="92"/>
     </row>
     <row r="403" ht="11.25" customHeight="1">
-      <c r="B403" s="95"/>
+      <c r="B403" s="92"/>
     </row>
     <row r="404" ht="11.25" customHeight="1">
-      <c r="B404" s="95"/>
+      <c r="B404" s="92"/>
     </row>
     <row r="405" ht="11.25" customHeight="1">
-      <c r="B405" s="95"/>
+      <c r="B405" s="92"/>
     </row>
     <row r="406" ht="11.25" customHeight="1">
-      <c r="B406" s="95"/>
+      <c r="B406" s="92"/>
     </row>
     <row r="407" ht="11.25" customHeight="1">
-      <c r="B407" s="95"/>
+      <c r="B407" s="92"/>
     </row>
     <row r="408" ht="11.25" customHeight="1">
-      <c r="B408" s="95"/>
+      <c r="B408" s="92"/>
     </row>
     <row r="409" ht="11.25" customHeight="1">
-      <c r="B409" s="95"/>
+      <c r="B409" s="92"/>
     </row>
     <row r="410" ht="11.25" customHeight="1">
-      <c r="B410" s="95"/>
+      <c r="B410" s="92"/>
     </row>
     <row r="411" ht="11.25" customHeight="1">
-      <c r="B411" s="95"/>
+      <c r="B411" s="92"/>
     </row>
     <row r="412" ht="11.25" customHeight="1">
-      <c r="B412" s="95"/>
+      <c r="B412" s="92"/>
     </row>
     <row r="413" ht="11.25" customHeight="1">
-      <c r="B413" s="95"/>
+      <c r="B413" s="92"/>
     </row>
     <row r="414" ht="11.25" customHeight="1">
-      <c r="B414" s="95"/>
+      <c r="B414" s="92"/>
     </row>
     <row r="415" ht="11.25" customHeight="1">
-      <c r="B415" s="95"/>
+      <c r="B415" s="92"/>
     </row>
     <row r="416" ht="11.25" customHeight="1">
-      <c r="B416" s="95"/>
+      <c r="B416" s="92"/>
     </row>
     <row r="417" ht="11.25" customHeight="1">
-      <c r="B417" s="95"/>
+      <c r="B417" s="92"/>
     </row>
     <row r="418" ht="11.25" customHeight="1">
-      <c r="B418" s="95"/>
+      <c r="B418" s="92"/>
     </row>
     <row r="419" ht="11.25" customHeight="1">
-      <c r="B419" s="95"/>
+      <c r="B419" s="92"/>
     </row>
     <row r="420" ht="11.25" customHeight="1">
-      <c r="B420" s="95"/>
+      <c r="B420" s="92"/>
     </row>
     <row r="421" ht="11.25" customHeight="1">
-      <c r="B421" s="95"/>
+      <c r="B421" s="92"/>
     </row>
     <row r="422" ht="11.25" customHeight="1">
-      <c r="B422" s="95"/>
+      <c r="B422" s="92"/>
     </row>
     <row r="423" ht="11.25" customHeight="1">
-      <c r="B423" s="95"/>
+      <c r="B423" s="92"/>
     </row>
     <row r="424" ht="11.25" customHeight="1">
-      <c r="B424" s="95"/>
+      <c r="B424" s="92"/>
     </row>
     <row r="425" ht="11.25" customHeight="1">
-      <c r="B425" s="95"/>
+      <c r="B425" s="92"/>
     </row>
     <row r="426" ht="11.25" customHeight="1">
-      <c r="B426" s="95"/>
+      <c r="B426" s="92"/>
     </row>
     <row r="427" ht="11.25" customHeight="1">
-      <c r="B427" s="95"/>
+      <c r="B427" s="92"/>
     </row>
     <row r="428" ht="11.25" customHeight="1">
-      <c r="B428" s="95"/>
+      <c r="B428" s="92"/>
     </row>
     <row r="429" ht="11.25" customHeight="1">
-      <c r="B429" s="95"/>
+      <c r="B429" s="92"/>
     </row>
     <row r="430" ht="11.25" customHeight="1">
-      <c r="B430" s="95"/>
+      <c r="B430" s="92"/>
     </row>
     <row r="431" ht="11.25" customHeight="1">
-      <c r="B431" s="95"/>
+      <c r="B431" s="92"/>
     </row>
     <row r="432" ht="11.25" customHeight="1">
-      <c r="B432" s="95"/>
+      <c r="B432" s="92"/>
     </row>
     <row r="433" ht="11.25" customHeight="1">
-      <c r="B433" s="95"/>
+      <c r="B433" s="92"/>
     </row>
     <row r="434" ht="11.25" customHeight="1">
-      <c r="B434" s="95"/>
+      <c r="B434" s="92"/>
     </row>
     <row r="435" ht="11.25" customHeight="1">
-      <c r="B435" s="95"/>
+      <c r="B435" s="92"/>
     </row>
     <row r="436" ht="11.25" customHeight="1">
-      <c r="B436" s="95"/>
+      <c r="B436" s="92"/>
     </row>
     <row r="437" ht="11.25" customHeight="1">
-      <c r="B437" s="95"/>
+      <c r="B437" s="92"/>
     </row>
     <row r="438" ht="11.25" customHeight="1">
-      <c r="B438" s="95"/>
+      <c r="B438" s="92"/>
     </row>
     <row r="439" ht="11.25" customHeight="1">
-      <c r="B439" s="95"/>
+      <c r="B439" s="92"/>
     </row>
     <row r="440" ht="11.25" customHeight="1">
-      <c r="B440" s="95"/>
+      <c r="B440" s="92"/>
     </row>
     <row r="441" ht="11.25" customHeight="1">
-      <c r="B441" s="95"/>
+      <c r="B441" s="92"/>
     </row>
     <row r="442" ht="11.25" customHeight="1">
-      <c r="B442" s="95"/>
+      <c r="B442" s="92"/>
     </row>
     <row r="443" ht="11.25" customHeight="1">
-      <c r="B443" s="95"/>
+      <c r="B443" s="92"/>
     </row>
     <row r="444" ht="11.25" customHeight="1">
-      <c r="B444" s="95"/>
+      <c r="B444" s="92"/>
     </row>
     <row r="445" ht="11.25" customHeight="1">
-      <c r="B445" s="95"/>
+      <c r="B445" s="92"/>
     </row>
     <row r="446" ht="11.25" customHeight="1">
-      <c r="B446" s="95"/>
+      <c r="B446" s="92"/>
     </row>
     <row r="447" ht="11.25" customHeight="1">
-      <c r="B447" s="95"/>
+      <c r="B447" s="92"/>
     </row>
     <row r="448" ht="11.25" customHeight="1">
-      <c r="B448" s="95"/>
+      <c r="B448" s="92"/>
     </row>
     <row r="449" ht="11.25" customHeight="1">
-      <c r="B449" s="95"/>
+      <c r="B449" s="92"/>
     </row>
     <row r="450" ht="11.25" customHeight="1">
-      <c r="B450" s="95"/>
+      <c r="B450" s="92"/>
     </row>
     <row r="451" ht="11.25" customHeight="1">
-      <c r="B451" s="95"/>
+      <c r="B451" s="92"/>
     </row>
     <row r="452" ht="11.25" customHeight="1">
-      <c r="B452" s="95"/>
+      <c r="B452" s="92"/>
     </row>
     <row r="453" ht="11.25" customHeight="1">
-      <c r="B453" s="95"/>
+      <c r="B453" s="92"/>
     </row>
     <row r="454" ht="11.25" customHeight="1">
-      <c r="B454" s="95"/>
+      <c r="B454" s="92"/>
     </row>
     <row r="455" ht="11.25" customHeight="1">
-      <c r="B455" s="95"/>
+      <c r="B455" s="92"/>
     </row>
     <row r="456" ht="11.25" customHeight="1">
-      <c r="B456" s="95"/>
+      <c r="B456" s="92"/>
     </row>
     <row r="457" ht="11.25" customHeight="1">
-      <c r="B457" s="95"/>
+      <c r="B457" s="92"/>
     </row>
     <row r="458" ht="11.25" customHeight="1">
-      <c r="B458" s="95"/>
+      <c r="B458" s="92"/>
     </row>
     <row r="459" ht="11.25" customHeight="1">
-      <c r="B459" s="95"/>
+      <c r="B459" s="92"/>
     </row>
     <row r="460" ht="11.25" customHeight="1">
-      <c r="B460" s="95"/>
+      <c r="B460" s="92"/>
     </row>
     <row r="461" ht="11.25" customHeight="1">
-      <c r="B461" s="95"/>
+      <c r="B461" s="92"/>
     </row>
     <row r="462" ht="11.25" customHeight="1">
-      <c r="B462" s="95"/>
+      <c r="B462" s="92"/>
     </row>
     <row r="463" ht="11.25" customHeight="1">
-      <c r="B463" s="95"/>
+      <c r="B463" s="92"/>
     </row>
     <row r="464" ht="11.25" customHeight="1">
-      <c r="B464" s="95"/>
+      <c r="B464" s="92"/>
     </row>
     <row r="465" ht="11.25" customHeight="1">
-      <c r="B465" s="95"/>
+      <c r="B465" s="92"/>
     </row>
     <row r="466" ht="11.25" customHeight="1">
-      <c r="B466" s="95"/>
+      <c r="B466" s="92"/>
     </row>
     <row r="467" ht="11.25" customHeight="1">
-      <c r="B467" s="95"/>
+      <c r="B467" s="92"/>
     </row>
     <row r="468" ht="11.25" customHeight="1">
-      <c r="B468" s="95"/>
+      <c r="B468" s="92"/>
     </row>
     <row r="469" ht="11.25" customHeight="1">
-      <c r="B469" s="95"/>
+      <c r="B469" s="92"/>
     </row>
     <row r="470" ht="11.25" customHeight="1">
-      <c r="B470" s="95"/>
+      <c r="B470" s="92"/>
     </row>
     <row r="471" ht="11.25" customHeight="1">
-      <c r="B471" s="95"/>
+      <c r="B471" s="92"/>
     </row>
     <row r="472" ht="11.25" customHeight="1">
-      <c r="B472" s="95"/>
+      <c r="B472" s="92"/>
     </row>
     <row r="473" ht="11.25" customHeight="1">
-      <c r="B473" s="95"/>
+      <c r="B473" s="92"/>
     </row>
     <row r="474" ht="11.25" customHeight="1">
-      <c r="B474" s="95"/>
+      <c r="B474" s="92"/>
     </row>
     <row r="475" ht="11.25" customHeight="1">
-      <c r="B475" s="95"/>
+      <c r="B475" s="92"/>
     </row>
     <row r="476" ht="11.25" customHeight="1">
-      <c r="B476" s="95"/>
+      <c r="B476" s="92"/>
     </row>
     <row r="477" ht="11.25" customHeight="1">
-      <c r="B477" s="95"/>
+      <c r="B477" s="92"/>
     </row>
     <row r="478" ht="11.25" customHeight="1">
-      <c r="B478" s="95"/>
+      <c r="B478" s="92"/>
     </row>
     <row r="479" ht="11.25" customHeight="1">
-      <c r="B479" s="95"/>
+      <c r="B479" s="92"/>
     </row>
     <row r="480" ht="11.25" customHeight="1">
-      <c r="B480" s="95"/>
+      <c r="B480" s="92"/>
     </row>
     <row r="481" ht="11.25" customHeight="1">
-      <c r="B481" s="95"/>
+      <c r="B481" s="92"/>
     </row>
     <row r="482" ht="11.25" customHeight="1">
-      <c r="B482" s="95"/>
+      <c r="B482" s="92"/>
     </row>
     <row r="483" ht="11.25" customHeight="1">
-      <c r="B483" s="95"/>
+      <c r="B483" s="92"/>
     </row>
     <row r="484" ht="11.25" customHeight="1">
-      <c r="B484" s="95"/>
+      <c r="B484" s="92"/>
     </row>
     <row r="485" ht="11.25" customHeight="1">
-      <c r="B485" s="95"/>
+      <c r="B485" s="92"/>
     </row>
     <row r="486" ht="11.25" customHeight="1">
-      <c r="B486" s="95"/>
+      <c r="B486" s="92"/>
     </row>
     <row r="487" ht="11.25" customHeight="1">
-      <c r="B487" s="95"/>
+      <c r="B487" s="92"/>
     </row>
     <row r="488" ht="11.25" customHeight="1">
-      <c r="B488" s="95"/>
+      <c r="B488" s="92"/>
     </row>
     <row r="489" ht="11.25" customHeight="1">
-      <c r="B489" s="95"/>
+      <c r="B489" s="92"/>
     </row>
     <row r="490" ht="11.25" customHeight="1">
-      <c r="B490" s="95"/>
+      <c r="B490" s="92"/>
     </row>
     <row r="491" ht="11.25" customHeight="1">
-      <c r="B491" s="95"/>
+      <c r="B491" s="92"/>
     </row>
     <row r="492" ht="11.25" customHeight="1">
-      <c r="B492" s="95"/>
+      <c r="B492" s="92"/>
     </row>
     <row r="493" ht="11.25" customHeight="1">
-      <c r="B493" s="95"/>
+      <c r="B493" s="92"/>
     </row>
     <row r="494" ht="11.25" customHeight="1">
-      <c r="B494" s="95"/>
+      <c r="B494" s="92"/>
     </row>
     <row r="495" ht="11.25" customHeight="1">
-      <c r="B495" s="95"/>
+      <c r="B495" s="92"/>
     </row>
     <row r="496" ht="11.25" customHeight="1">
-      <c r="B496" s="95"/>
+      <c r="B496" s="92"/>
     </row>
     <row r="497" ht="11.25" customHeight="1">
-      <c r="B497" s="95"/>
+      <c r="B497" s="92"/>
     </row>
     <row r="498" ht="11.25" customHeight="1">
-      <c r="B498" s="95"/>
+      <c r="B498" s="92"/>
     </row>
     <row r="499" ht="11.25" customHeight="1">
-      <c r="B499" s="95"/>
+      <c r="B499" s="92"/>
     </row>
     <row r="500" ht="11.25" customHeight="1">
-      <c r="B500" s="95"/>
+      <c r="B500" s="92"/>
     </row>
     <row r="501" ht="11.25" customHeight="1">
-      <c r="B501" s="95"/>
+      <c r="B501" s="92"/>
     </row>
     <row r="502" ht="11.25" customHeight="1">
-      <c r="B502" s="95"/>
+      <c r="B502" s="92"/>
     </row>
     <row r="503" ht="11.25" customHeight="1">
-      <c r="B503" s="95"/>
+      <c r="B503" s="92"/>
     </row>
     <row r="504" ht="11.25" customHeight="1">
-      <c r="B504" s="95"/>
+      <c r="B504" s="92"/>
     </row>
     <row r="505" ht="11.25" customHeight="1">
-      <c r="B505" s="95"/>
+      <c r="B505" s="92"/>
     </row>
     <row r="506" ht="11.25" customHeight="1">
-      <c r="B506" s="95"/>
+      <c r="B506" s="92"/>
     </row>
     <row r="507" ht="11.25" customHeight="1">
-      <c r="B507" s="95"/>
+      <c r="B507" s="92"/>
     </row>
     <row r="508" ht="11.25" customHeight="1">
-      <c r="B508" s="95"/>
+      <c r="B508" s="92"/>
     </row>
     <row r="509" ht="11.25" customHeight="1">
-      <c r="B509" s="95"/>
+      <c r="B509" s="92"/>
     </row>
     <row r="510" ht="11.25" customHeight="1">
-      <c r="B510" s="95"/>
+      <c r="B510" s="92"/>
     </row>
     <row r="511" ht="11.25" customHeight="1">
-      <c r="B511" s="95"/>
+      <c r="B511" s="92"/>
     </row>
     <row r="512" ht="11.25" customHeight="1">
-      <c r="B512" s="95"/>
+      <c r="B512" s="92"/>
     </row>
     <row r="513" ht="11.25" customHeight="1">
-      <c r="B513" s="95"/>
+      <c r="B513" s="92"/>
     </row>
     <row r="514" ht="11.25" customHeight="1">
-      <c r="B514" s="95"/>
+      <c r="B514" s="92"/>
     </row>
     <row r="515" ht="11.25" customHeight="1">
-      <c r="B515" s="95"/>
+      <c r="B515" s="92"/>
     </row>
     <row r="516" ht="11.25" customHeight="1">
-      <c r="B516" s="95"/>
+      <c r="B516" s="92"/>
     </row>
     <row r="517" ht="11.25" customHeight="1">
-      <c r="B517" s="95"/>
+      <c r="B517" s="92"/>
     </row>
     <row r="518" ht="11.25" customHeight="1">
-      <c r="B518" s="95"/>
+      <c r="B518" s="92"/>
     </row>
     <row r="519" ht="11.25" customHeight="1">
-      <c r="B519" s="95"/>
+      <c r="B519" s="92"/>
     </row>
     <row r="520" ht="11.25" customHeight="1">
-      <c r="B520" s="95"/>
+      <c r="B520" s="92"/>
     </row>
     <row r="521" ht="11.25" customHeight="1">
-      <c r="B521" s="95"/>
+      <c r="B521" s="92"/>
     </row>
     <row r="522" ht="11.25" customHeight="1">
-      <c r="B522" s="95"/>
+      <c r="B522" s="92"/>
     </row>
     <row r="523" ht="11.25" customHeight="1">
-      <c r="B523" s="95"/>
+      <c r="B523" s="92"/>
     </row>
     <row r="524" ht="11.25" customHeight="1">
-      <c r="B524" s="95"/>
+      <c r="B524" s="92"/>
     </row>
     <row r="525" ht="11.25" customHeight="1">
-      <c r="B525" s="95"/>
+      <c r="B525" s="92"/>
     </row>
     <row r="526" ht="11.25" customHeight="1">
-      <c r="B526" s="95"/>
+      <c r="B526" s="92"/>
     </row>
     <row r="527" ht="11.25" customHeight="1">
-      <c r="B527" s="95"/>
+      <c r="B527" s="92"/>
     </row>
     <row r="528" ht="11.25" customHeight="1">
-      <c r="B528" s="95"/>
+      <c r="B528" s="92"/>
     </row>
     <row r="529" ht="11.25" customHeight="1">
-      <c r="B529" s="95"/>
+      <c r="B529" s="92"/>
     </row>
     <row r="530" ht="11.25" customHeight="1">
-      <c r="B530" s="95"/>
+      <c r="B530" s="92"/>
     </row>
     <row r="531" ht="11.25" customHeight="1">
-      <c r="B531" s="95"/>
+      <c r="B531" s="92"/>
     </row>
     <row r="532" ht="11.25" customHeight="1">
-      <c r="B532" s="95"/>
+      <c r="B532" s="92"/>
     </row>
     <row r="533" ht="11.25" customHeight="1">
-      <c r="B533" s="95"/>
+      <c r="B533" s="92"/>
     </row>
     <row r="534" ht="11.25" customHeight="1">
-      <c r="B534" s="95"/>
+      <c r="B534" s="92"/>
     </row>
     <row r="535" ht="11.25" customHeight="1">
-      <c r="B535" s="95"/>
+      <c r="B535" s="92"/>
     </row>
     <row r="536" ht="11.25" customHeight="1">
-      <c r="B536" s="95"/>
+      <c r="B536" s="92"/>
     </row>
     <row r="537" ht="11.25" customHeight="1">
-      <c r="B537" s="95"/>
+      <c r="B537" s="92"/>
     </row>
     <row r="538" ht="11.25" customHeight="1">
-      <c r="B538" s="95"/>
+      <c r="B538" s="92"/>
     </row>
     <row r="539" ht="11.25" customHeight="1">
-      <c r="B539" s="95"/>
+      <c r="B539" s="92"/>
     </row>
     <row r="540" ht="11.25" customHeight="1">
-      <c r="B540" s="95"/>
+      <c r="B540" s="92"/>
     </row>
     <row r="541" ht="11.25" customHeight="1">
-      <c r="B541" s="95"/>
+      <c r="B541" s="92"/>
     </row>
     <row r="542" ht="11.25" customHeight="1">
-      <c r="B542" s="95"/>
+      <c r="B542" s="92"/>
     </row>
     <row r="543" ht="11.25" customHeight="1">
-      <c r="B543" s="95"/>
+      <c r="B543" s="92"/>
     </row>
     <row r="544" ht="11.25" customHeight="1">
-      <c r="B544" s="95"/>
+      <c r="B544" s="92"/>
     </row>
     <row r="545" ht="11.25" customHeight="1">
-      <c r="B545" s="95"/>
+      <c r="B545" s="92"/>
     </row>
     <row r="546" ht="11.25" customHeight="1">
-      <c r="B546" s="95"/>
+      <c r="B546" s="92"/>
     </row>
     <row r="547" ht="11.25" customHeight="1">
-      <c r="B547" s="95"/>
+      <c r="B547" s="92"/>
     </row>
     <row r="548" ht="11.25" customHeight="1">
-      <c r="B548" s="95"/>
+      <c r="B548" s="92"/>
     </row>
     <row r="549" ht="11.25" customHeight="1">
-      <c r="B549" s="95"/>
+      <c r="B549" s="92"/>
     </row>
     <row r="550" ht="11.25" customHeight="1">
-      <c r="B550" s="95"/>
+      <c r="B550" s="92"/>
     </row>
     <row r="551" ht="11.25" customHeight="1">
-      <c r="B551" s="95"/>
+      <c r="B551" s="92"/>
     </row>
     <row r="552" ht="11.25" customHeight="1">
-      <c r="B552" s="95"/>
+      <c r="B552" s="92"/>
     </row>
     <row r="553" ht="11.25" customHeight="1">
-      <c r="B553" s="95"/>
+      <c r="B553" s="92"/>
     </row>
     <row r="554" ht="11.25" customHeight="1">
-      <c r="B554" s="95"/>
+      <c r="B554" s="92"/>
     </row>
     <row r="555" ht="11.25" customHeight="1">
-      <c r="B555" s="95"/>
+      <c r="B555" s="92"/>
     </row>
     <row r="556" ht="11.25" customHeight="1">
-      <c r="B556" s="95"/>
+      <c r="B556" s="92"/>
     </row>
     <row r="557" ht="11.25" customHeight="1">
-      <c r="B557" s="95"/>
+      <c r="B557" s="92"/>
     </row>
     <row r="558" ht="11.25" customHeight="1">
-      <c r="B558" s="95"/>
+      <c r="B558" s="92"/>
     </row>
     <row r="559" ht="11.25" customHeight="1">
-      <c r="B559" s="95"/>
+      <c r="B559" s="92"/>
     </row>
     <row r="560" ht="11.25" customHeight="1">
-      <c r="B560" s="95"/>
+      <c r="B560" s="92"/>
     </row>
     <row r="561" ht="11.25" customHeight="1">
-      <c r="B561" s="95"/>
+      <c r="B561" s="92"/>
     </row>
     <row r="562" ht="11.25" customHeight="1">
-      <c r="B562" s="95"/>
+      <c r="B562" s="92"/>
     </row>
     <row r="563" ht="11.25" customHeight="1">
-      <c r="B563" s="95"/>
+      <c r="B563" s="92"/>
     </row>
     <row r="564" ht="11.25" customHeight="1">
-      <c r="B564" s="95"/>
+      <c r="B564" s="92"/>
     </row>
     <row r="565" ht="11.25" customHeight="1">
-      <c r="B565" s="95"/>
+      <c r="B565" s="92"/>
     </row>
     <row r="566" ht="11.25" customHeight="1">
-      <c r="B566" s="95"/>
+      <c r="B566" s="92"/>
     </row>
     <row r="567" ht="11.25" customHeight="1">
-      <c r="B567" s="95"/>
+      <c r="B567" s="92"/>
     </row>
     <row r="568" ht="11.25" customHeight="1">
-      <c r="B568" s="95"/>
+      <c r="B568" s="92"/>
     </row>
     <row r="569" ht="11.25" customHeight="1">
-      <c r="B569" s="95"/>
+      <c r="B569" s="92"/>
     </row>
     <row r="570" ht="11.25" customHeight="1">
-      <c r="B570" s="95"/>
+      <c r="B570" s="92"/>
     </row>
     <row r="571" ht="11.25" customHeight="1">
-      <c r="B571" s="95"/>
+      <c r="B571" s="92"/>
     </row>
     <row r="572" ht="11.25" customHeight="1">
-      <c r="B572" s="95"/>
+      <c r="B572" s="92"/>
     </row>
     <row r="573" ht="11.25" customHeight="1">
-      <c r="B573" s="95"/>
+      <c r="B573" s="92"/>
     </row>
     <row r="574" ht="11.25" customHeight="1">
-      <c r="B574" s="95"/>
+      <c r="B574" s="92"/>
     </row>
     <row r="575" ht="11.25" customHeight="1">
-      <c r="B575" s="95"/>
+      <c r="B575" s="92"/>
     </row>
     <row r="576" ht="11.25" customHeight="1">
-      <c r="B576" s="95"/>
+      <c r="B576" s="92"/>
     </row>
     <row r="577" ht="11.25" customHeight="1">
-      <c r="B577" s="95"/>
+      <c r="B577" s="92"/>
     </row>
     <row r="578" ht="11.25" customHeight="1">
-      <c r="B578" s="95"/>
+      <c r="B578" s="92"/>
     </row>
     <row r="579" ht="11.25" customHeight="1">
-      <c r="B579" s="95"/>
+      <c r="B579" s="92"/>
     </row>
     <row r="580" ht="11.25" customHeight="1">
-      <c r="B580" s="95"/>
+      <c r="B580" s="92"/>
     </row>
     <row r="581" ht="11.25" customHeight="1">
-      <c r="B581" s="95"/>
+      <c r="B581" s="92"/>
     </row>
     <row r="582" ht="11.25" customHeight="1">
-      <c r="B582" s="95"/>
+      <c r="B582" s="92"/>
     </row>
     <row r="583" ht="11.25" customHeight="1">
-      <c r="B583" s="95"/>
+      <c r="B583" s="92"/>
     </row>
     <row r="584" ht="11.25" customHeight="1">
-      <c r="B584" s="95"/>
+      <c r="B584" s="92"/>
     </row>
     <row r="585" ht="11.25" customHeight="1">
-      <c r="B585" s="95"/>
+      <c r="B585" s="92"/>
     </row>
     <row r="586" ht="11.25" customHeight="1">
-      <c r="B586" s="95"/>
+      <c r="B586" s="92"/>
     </row>
     <row r="587" ht="11.25" customHeight="1">
-      <c r="B587" s="95"/>
+      <c r="B587" s="92"/>
     </row>
     <row r="588" ht="11.25" customHeight="1">
-      <c r="B588" s="95"/>
+      <c r="B588" s="92"/>
     </row>
     <row r="589" ht="11.25" customHeight="1">
-      <c r="B589" s="95"/>
+      <c r="B589" s="92"/>
     </row>
     <row r="590" ht="11.25" customHeight="1">
-      <c r="B590" s="95"/>
+      <c r="B590" s="92"/>
     </row>
     <row r="591" ht="11.25" customHeight="1">
-      <c r="B591" s="95"/>
+      <c r="B591" s="92"/>
     </row>
     <row r="592" ht="11.25" customHeight="1">
-      <c r="B592" s="95"/>
+      <c r="B592" s="92"/>
     </row>
     <row r="593" ht="11.25" customHeight="1">
-      <c r="B593" s="95"/>
+      <c r="B593" s="92"/>
     </row>
     <row r="594" ht="11.25" customHeight="1">
-      <c r="B594" s="95"/>
+      <c r="B594" s="92"/>
     </row>
     <row r="595" ht="11.25" customHeight="1">
-      <c r="B595" s="95"/>
+      <c r="B595" s="92"/>
     </row>
     <row r="596" ht="11.25" customHeight="1">
-      <c r="B596" s="95"/>
+      <c r="B596" s="92"/>
     </row>
     <row r="597" ht="11.25" customHeight="1">
-      <c r="B597" s="95"/>
+      <c r="B597" s="92"/>
     </row>
     <row r="598" ht="11.25" customHeight="1">
-      <c r="B598" s="95"/>
+      <c r="B598" s="92"/>
     </row>
     <row r="599" ht="11.25" customHeight="1">
-      <c r="B599" s="95"/>
+      <c r="B599" s="92"/>
     </row>
     <row r="600" ht="11.25" customHeight="1">
-      <c r="B600" s="95"/>
+      <c r="B600" s="92"/>
     </row>
     <row r="601" ht="11.25" customHeight="1">
-      <c r="B601" s="95"/>
+      <c r="B601" s="92"/>
     </row>
     <row r="602" ht="11.25" customHeight="1">
-      <c r="B602" s="95"/>
+      <c r="B602" s="92"/>
     </row>
     <row r="603" ht="11.25" customHeight="1">
-      <c r="B603" s="95"/>
+      <c r="B603" s="92"/>
     </row>
     <row r="604" ht="11.25" customHeight="1">
-      <c r="B604" s="95"/>
+      <c r="B604" s="92"/>
     </row>
     <row r="605" ht="11.25" customHeight="1">
-      <c r="B605" s="95"/>
+      <c r="B605" s="92"/>
     </row>
     <row r="606" ht="11.25" customHeight="1">
-      <c r="B606" s="95"/>
+      <c r="B606" s="92"/>
     </row>
     <row r="607" ht="11.25" customHeight="1">
-      <c r="B607" s="95"/>
+      <c r="B607" s="92"/>
     </row>
     <row r="608" ht="11.25" customHeight="1">
-      <c r="B608" s="95"/>
+      <c r="B608" s="92"/>
     </row>
     <row r="609" ht="11.25" customHeight="1">
-      <c r="B609" s="95"/>
+      <c r="B609" s="92"/>
     </row>
     <row r="610" ht="11.25" customHeight="1">
-      <c r="B610" s="95"/>
+      <c r="B610" s="92"/>
     </row>
     <row r="611" ht="11.25" customHeight="1">
-      <c r="B611" s="95"/>
+      <c r="B611" s="92"/>
     </row>
     <row r="612" ht="11.25" customHeight="1">
-      <c r="B612" s="95"/>
+      <c r="B612" s="92"/>
     </row>
     <row r="613" ht="11.25" customHeight="1">
-      <c r="B613" s="95"/>
+      <c r="B613" s="92"/>
     </row>
     <row r="614" ht="11.25" customHeight="1">
-      <c r="B614" s="95"/>
+      <c r="B614" s="92"/>
     </row>
     <row r="615" ht="11.25" customHeight="1">
-      <c r="B615" s="95"/>
+      <c r="B615" s="92"/>
     </row>
     <row r="616" ht="11.25" customHeight="1">
-      <c r="B616" s="95"/>
+      <c r="B616" s="92"/>
     </row>
     <row r="617" ht="11.25" customHeight="1">
-      <c r="B617" s="95"/>
+      <c r="B617" s="92"/>
     </row>
     <row r="618" ht="11.25" customHeight="1">
-      <c r="B618" s="95"/>
+      <c r="B618" s="92"/>
     </row>
     <row r="619" ht="11.25" customHeight="1">
-      <c r="B619" s="95"/>
+      <c r="B619" s="92"/>
     </row>
     <row r="620" ht="11.25" customHeight="1">
-      <c r="B620" s="95"/>
+      <c r="B620" s="92"/>
     </row>
     <row r="621" ht="11.25" customHeight="1">
-      <c r="B621" s="95"/>
+      <c r="B621" s="92"/>
     </row>
     <row r="622" ht="11.25" customHeight="1">
-      <c r="B622" s="95"/>
+      <c r="B622" s="92"/>
     </row>
     <row r="623" ht="11.25" customHeight="1">
-      <c r="B623" s="95"/>
+      <c r="B623" s="92"/>
     </row>
     <row r="624" ht="11.25" customHeight="1">
-      <c r="B624" s="95"/>
+      <c r="B624" s="92"/>
     </row>
     <row r="625" ht="11.25" customHeight="1">
-      <c r="B625" s="95"/>
+      <c r="B625" s="92"/>
     </row>
     <row r="626" ht="11.25" customHeight="1">
-      <c r="B626" s="95"/>
+      <c r="B626" s="92"/>
     </row>
     <row r="627" ht="11.25" customHeight="1">
-      <c r="B627" s="95"/>
+      <c r="B627" s="92"/>
     </row>
     <row r="628" ht="11.25" customHeight="1">
-      <c r="B628" s="95"/>
+      <c r="B628" s="92"/>
     </row>
     <row r="629" ht="11.25" customHeight="1">
-      <c r="B629" s="95"/>
+      <c r="B629" s="92"/>
     </row>
     <row r="630" ht="11.25" customHeight="1">
-      <c r="B630" s="95"/>
+      <c r="B630" s="92"/>
     </row>
     <row r="631" ht="11.25" customHeight="1">
-      <c r="B631" s="95"/>
+      <c r="B631" s="92"/>
     </row>
     <row r="632" ht="11.25" customHeight="1">
-      <c r="B632" s="95"/>
+      <c r="B632" s="92"/>
     </row>
     <row r="633" ht="11.25" customHeight="1">
-      <c r="B633" s="95"/>
+      <c r="B633" s="92"/>
     </row>
     <row r="634" ht="11.25" customHeight="1">
-      <c r="B634" s="95"/>
+      <c r="B634" s="92"/>
     </row>
     <row r="635" ht="11.25" customHeight="1">
-      <c r="B635" s="95"/>
+      <c r="B635" s="92"/>
     </row>
     <row r="636" ht="11.25" customHeight="1">
-      <c r="B636" s="95"/>
+      <c r="B636" s="92"/>
     </row>
     <row r="637" ht="11.25" customHeight="1">
-      <c r="B637" s="95"/>
+      <c r="B637" s="92"/>
     </row>
     <row r="638" ht="11.25" customHeight="1">
-      <c r="B638" s="95"/>
+      <c r="B638" s="92"/>
     </row>
     <row r="639" ht="11.25" customHeight="1">
-      <c r="B639" s="95"/>
+      <c r="B639" s="92"/>
     </row>
     <row r="640" ht="11.25" customHeight="1">
-      <c r="B640" s="95"/>
+      <c r="B640" s="92"/>
     </row>
     <row r="641" ht="11.25" customHeight="1">
-      <c r="B641" s="95"/>
+      <c r="B641" s="92"/>
     </row>
     <row r="642" ht="11.25" customHeight="1">
-      <c r="B642" s="95"/>
+      <c r="B642" s="92"/>
     </row>
     <row r="643" ht="11.25" customHeight="1">
-      <c r="B643" s="95"/>
+      <c r="B643" s="92"/>
     </row>
     <row r="644" ht="11.25" customHeight="1">
-      <c r="B644" s="95"/>
+      <c r="B644" s="92"/>
     </row>
     <row r="645" ht="11.25" customHeight="1">
-      <c r="B645" s="95"/>
+      <c r="B645" s="92"/>
     </row>
     <row r="646" ht="11.25" customHeight="1">
-      <c r="B646" s="95"/>
+      <c r="B646" s="92"/>
     </row>
     <row r="647" ht="11.25" customHeight="1">
-      <c r="B647" s="95"/>
+      <c r="B647" s="92"/>
     </row>
     <row r="648" ht="11.25" customHeight="1">
-      <c r="B648" s="95"/>
+      <c r="B648" s="92"/>
     </row>
     <row r="649" ht="11.25" customHeight="1">
-      <c r="B649" s="95"/>
+      <c r="B649" s="92"/>
     </row>
     <row r="650" ht="11.25" customHeight="1">
-      <c r="B650" s="95"/>
+      <c r="B650" s="92"/>
     </row>
     <row r="651" ht="11.25" customHeight="1">
-      <c r="B651" s="95"/>
+      <c r="B651" s="92"/>
     </row>
     <row r="652" ht="11.25" customHeight="1">
-      <c r="B652" s="95"/>
+      <c r="B652" s="92"/>
     </row>
     <row r="653" ht="11.25" customHeight="1">
-      <c r="B653" s="95"/>
+      <c r="B653" s="92"/>
     </row>
     <row r="654" ht="11.25" customHeight="1">
-      <c r="B654" s="95"/>
+      <c r="B654" s="92"/>
     </row>
     <row r="655" ht="11.25" customHeight="1">
-      <c r="B655" s="95"/>
+      <c r="B655" s="92"/>
     </row>
     <row r="656" ht="11.25" customHeight="1">
-      <c r="B656" s="95"/>
+      <c r="B656" s="92"/>
     </row>
     <row r="657" ht="11.25" customHeight="1">
-      <c r="B657" s="95"/>
+      <c r="B657" s="92"/>
     </row>
     <row r="658" ht="11.25" customHeight="1">
-      <c r="B658" s="95"/>
+      <c r="B658" s="92"/>
     </row>
     <row r="659" ht="11.25" customHeight="1">
-      <c r="B659" s="95"/>
+      <c r="B659" s="92"/>
     </row>
     <row r="660" ht="11.25" customHeight="1">
-      <c r="B660" s="95"/>
+      <c r="B660" s="92"/>
     </row>
     <row r="661" ht="11.25" customHeight="1">
-      <c r="B661" s="95"/>
+      <c r="B661" s="92"/>
     </row>
     <row r="662" ht="11.25" customHeight="1">
-      <c r="B662" s="95"/>
+      <c r="B662" s="92"/>
     </row>
     <row r="663" ht="11.25" customHeight="1">
-      <c r="B663" s="95"/>
+      <c r="B663" s="92"/>
     </row>
     <row r="664" ht="11.25" customHeight="1">
-      <c r="B664" s="95"/>
+      <c r="B664" s="92"/>
     </row>
     <row r="665" ht="11.25" customHeight="1">
-      <c r="B665" s="95"/>
+      <c r="B665" s="92"/>
     </row>
     <row r="666" ht="11.25" customHeight="1">
-      <c r="B666" s="95"/>
+      <c r="B666" s="92"/>
     </row>
     <row r="667" ht="11.25" customHeight="1">
-      <c r="B667" s="95"/>
+      <c r="B667" s="92"/>
     </row>
     <row r="668" ht="11.25" customHeight="1">
-      <c r="B668" s="95"/>
+      <c r="B668" s="92"/>
     </row>
     <row r="669" ht="11.25" customHeight="1">
-      <c r="B669" s="95"/>
+      <c r="B669" s="92"/>
     </row>
     <row r="670" ht="11.25" customHeight="1">
-      <c r="B670" s="95"/>
+      <c r="B670" s="92"/>
     </row>
     <row r="671" ht="11.25" customHeight="1">
-      <c r="B671" s="95"/>
+      <c r="B671" s="92"/>
     </row>
     <row r="672" ht="11.25" customHeight="1">
-      <c r="B672" s="95"/>
+      <c r="B672" s="92"/>
     </row>
     <row r="673" ht="11.25" customHeight="1">
-      <c r="B673" s="95"/>
+      <c r="B673" s="92"/>
     </row>
     <row r="674" ht="11.25" customHeight="1">
-      <c r="B674" s="95"/>
+      <c r="B674" s="92"/>
     </row>
     <row r="675" ht="11.25" customHeight="1">
-      <c r="B675" s="95"/>
+      <c r="B675" s="92"/>
     </row>
     <row r="676" ht="11.25" customHeight="1">
-      <c r="B676" s="95"/>
+      <c r="B676" s="92"/>
     </row>
     <row r="677" ht="11.25" customHeight="1">
-      <c r="B677" s="95"/>
+      <c r="B677" s="92"/>
     </row>
     <row r="678" ht="11.25" customHeight="1">
-      <c r="B678" s="95"/>
+      <c r="B678" s="92"/>
     </row>
     <row r="679" ht="11.25" customHeight="1">
-      <c r="B679" s="95"/>
+      <c r="B679" s="92"/>
     </row>
     <row r="680" ht="11.25" customHeight="1">
-      <c r="B680" s="95"/>
+      <c r="B680" s="92"/>
     </row>
     <row r="681" ht="11.25" customHeight="1">
-      <c r="B681" s="95"/>
+      <c r="B681" s="92"/>
     </row>
     <row r="682" ht="11.25" customHeight="1">
-      <c r="B682" s="95"/>
+      <c r="B682" s="92"/>
     </row>
     <row r="683" ht="11.25" customHeight="1">
-      <c r="B683" s="95"/>
+      <c r="B683" s="92"/>
     </row>
     <row r="684" ht="11.25" customHeight="1">
-      <c r="B684" s="95"/>
+      <c r="B684" s="92"/>
     </row>
     <row r="685" ht="11.25" customHeight="1">
-      <c r="B685" s="95"/>
+      <c r="B685" s="92"/>
     </row>
     <row r="686" ht="11.25" customHeight="1">
-      <c r="B686" s="95"/>
+      <c r="B686" s="92"/>
     </row>
     <row r="687" ht="11.25" customHeight="1">
-      <c r="B687" s="95"/>
+      <c r="B687" s="92"/>
     </row>
     <row r="688" ht="11.25" customHeight="1">
-      <c r="B688" s="95"/>
+      <c r="B688" s="92"/>
     </row>
     <row r="689" ht="11.25" customHeight="1">
-      <c r="B689" s="95"/>
+      <c r="B689" s="92"/>
     </row>
     <row r="690" ht="11.25" customHeight="1">
-      <c r="B690" s="95"/>
+      <c r="B690" s="92"/>
     </row>
     <row r="691" ht="11.25" customHeight="1">
-      <c r="B691" s="95"/>
+      <c r="B691" s="92"/>
     </row>
     <row r="692" ht="11.25" customHeight="1">
-      <c r="B692" s="95"/>
+      <c r="B692" s="92"/>
     </row>
     <row r="693" ht="11.25" customHeight="1">
-      <c r="B693" s="95"/>
+      <c r="B693" s="92"/>
     </row>
     <row r="694" ht="11.25" customHeight="1">
-      <c r="B694" s="95"/>
+      <c r="B694" s="92"/>
     </row>
     <row r="695" ht="11.25" customHeight="1">
-      <c r="B695" s="95"/>
+      <c r="B695" s="92"/>
     </row>
     <row r="696" ht="11.25" customHeight="1">
-      <c r="B696" s="95"/>
+      <c r="B696" s="92"/>
     </row>
     <row r="697" ht="11.25" customHeight="1">
-      <c r="B697" s="95"/>
+      <c r="B697" s="92"/>
     </row>
     <row r="698" ht="11.25" customHeight="1">
-      <c r="B698" s="95"/>
+      <c r="B698" s="92"/>
     </row>
     <row r="699" ht="11.25" customHeight="1">
-      <c r="B699" s="95"/>
+      <c r="B699" s="92"/>
     </row>
     <row r="700" ht="11.25" customHeight="1">
-      <c r="B700" s="95"/>
+      <c r="B700" s="92"/>
     </row>
     <row r="701" ht="11.25" customHeight="1">
-      <c r="B701" s="95"/>
+      <c r="B701" s="92"/>
     </row>
     <row r="702" ht="11.25" customHeight="1">
-      <c r="B702" s="95"/>
+      <c r="B702" s="92"/>
     </row>
     <row r="703" ht="11.25" customHeight="1">
-      <c r="B703" s="95"/>
+      <c r="B703" s="92"/>
     </row>
     <row r="704" ht="11.25" customHeight="1">
-      <c r="B704" s="95"/>
+      <c r="B704" s="92"/>
     </row>
     <row r="705" ht="11.25" customHeight="1">
-      <c r="B705" s="95"/>
+      <c r="B705" s="92"/>
     </row>
     <row r="706" ht="11.25" customHeight="1">
-      <c r="B706" s="95"/>
+      <c r="B706" s="92"/>
     </row>
     <row r="707" ht="11.25" customHeight="1">
-      <c r="B707" s="95"/>
+      <c r="B707" s="92"/>
     </row>
     <row r="708" ht="11.25" customHeight="1">
-      <c r="B708" s="95"/>
+      <c r="B708" s="92"/>
     </row>
     <row r="709" ht="11.25" customHeight="1">
-      <c r="B709" s="95"/>
+      <c r="B709" s="92"/>
     </row>
     <row r="710" ht="11.25" customHeight="1">
-      <c r="B710" s="95"/>
+      <c r="B710" s="92"/>
     </row>
     <row r="711" ht="11.25" customHeight="1">
-      <c r="B711" s="95"/>
+      <c r="B711" s="92"/>
     </row>
     <row r="712" ht="11.25" customHeight="1">
-      <c r="B712" s="95"/>
+      <c r="B712" s="92"/>
     </row>
     <row r="713" ht="11.25" customHeight="1">
-      <c r="B713" s="95"/>
+      <c r="B713" s="92"/>
     </row>
     <row r="714" ht="11.25" customHeight="1">
-      <c r="B714" s="95"/>
+      <c r="B714" s="92"/>
     </row>
     <row r="715" ht="11.25" customHeight="1">
-      <c r="B715" s="95"/>
+      <c r="B715" s="92"/>
     </row>
     <row r="716" ht="11.25" customHeight="1">
-      <c r="B716" s="95"/>
+      <c r="B716" s="92"/>
     </row>
     <row r="717" ht="11.25" customHeight="1">
-      <c r="B717" s="95"/>
+      <c r="B717" s="92"/>
     </row>
     <row r="718" ht="11.25" customHeight="1">
-      <c r="B718" s="95"/>
+      <c r="B718" s="92"/>
     </row>
     <row r="719" ht="11.25" customHeight="1">
-      <c r="B719" s="95"/>
+      <c r="B719" s="92"/>
     </row>
     <row r="720" ht="11.25" customHeight="1">
-      <c r="B720" s="95"/>
+      <c r="B720" s="92"/>
     </row>
     <row r="721" ht="11.25" customHeight="1">
-      <c r="B721" s="95"/>
+      <c r="B721" s="92"/>
     </row>
     <row r="722" ht="11.25" customHeight="1">
-      <c r="B722" s="95"/>
+      <c r="B722" s="92"/>
     </row>
     <row r="723" ht="11.25" customHeight="1">
-      <c r="B723" s="95"/>
+      <c r="B723" s="92"/>
     </row>
     <row r="724" ht="11.25" customHeight="1">
-      <c r="B724" s="95"/>
+      <c r="B724" s="92"/>
     </row>
     <row r="725" ht="11.25" customHeight="1">
-      <c r="B725" s="95"/>
+      <c r="B725" s="92"/>
     </row>
     <row r="726" ht="11.25" customHeight="1">
-      <c r="B726" s="95"/>
+      <c r="B726" s="92"/>
     </row>
     <row r="727" ht="11.25" customHeight="1">
-      <c r="B727" s="95"/>
+      <c r="B727" s="92"/>
     </row>
     <row r="728" ht="11.25" customHeight="1">
-      <c r="B728" s="95"/>
+      <c r="B728" s="92"/>
     </row>
     <row r="729" ht="11.25" customHeight="1">
-      <c r="B729" s="95"/>
+      <c r="B729" s="92"/>
     </row>
     <row r="730" ht="11.25" customHeight="1">
-      <c r="B730" s="95"/>
+      <c r="B730" s="92"/>
     </row>
     <row r="731" ht="11.25" customHeight="1">
-      <c r="B731" s="95"/>
+      <c r="B731" s="92"/>
     </row>
     <row r="732" ht="11.25" customHeight="1">
-      <c r="B732" s="95"/>
+      <c r="B732" s="92"/>
     </row>
     <row r="733" ht="11.25" customHeight="1">
-      <c r="B733" s="95"/>
+      <c r="B733" s="92"/>
     </row>
     <row r="734" ht="11.25" customHeight="1">
-      <c r="B734" s="95"/>
+      <c r="B734" s="92"/>
     </row>
     <row r="735" ht="11.25" customHeight="1">
-      <c r="B735" s="95"/>
+      <c r="B735" s="92"/>
     </row>
     <row r="736" ht="11.25" customHeight="1">
-      <c r="B736" s="95"/>
+      <c r="B736" s="92"/>
     </row>
     <row r="737" ht="11.25" customHeight="1">
-      <c r="B737" s="95"/>
+      <c r="B737" s="92"/>
     </row>
     <row r="738" ht="11.25" customHeight="1">
-      <c r="B738" s="95"/>
+      <c r="B738" s="92"/>
     </row>
     <row r="739" ht="11.25" customHeight="1">
-      <c r="B739" s="95"/>
+      <c r="B739" s="92"/>
     </row>
     <row r="740" ht="11.25" customHeight="1">
-      <c r="B740" s="95"/>
+      <c r="B740" s="92"/>
     </row>
     <row r="741" ht="11.25" customHeight="1">
-      <c r="B741" s="95"/>
+      <c r="B741" s="92"/>
     </row>
     <row r="742" ht="11.25" customHeight="1">
-      <c r="B742" s="95"/>
+      <c r="B742" s="92"/>
     </row>
     <row r="743" ht="11.25" customHeight="1">
-      <c r="B743" s="95"/>
+      <c r="B743" s="92"/>
     </row>
     <row r="744" ht="11.25" customHeight="1">
-      <c r="B744" s="95"/>
+      <c r="B744" s="92"/>
     </row>
     <row r="745" ht="11.25" customHeight="1">
-      <c r="B745" s="95"/>
+      <c r="B745" s="92"/>
     </row>
     <row r="746" ht="11.25" customHeight="1">
-      <c r="B746" s="95"/>
+      <c r="B746" s="92"/>
     </row>
     <row r="747" ht="11.25" customHeight="1">
-      <c r="B747" s="95"/>
+      <c r="B747" s="92"/>
     </row>
     <row r="748" ht="11.25" customHeight="1">
-      <c r="B748" s="95"/>
+      <c r="B748" s="92"/>
     </row>
     <row r="749" ht="11.25" customHeight="1">
-      <c r="B749" s="95"/>
+      <c r="B749" s="92"/>
     </row>
     <row r="750" ht="11.25" customHeight="1">
-      <c r="B750" s="95"/>
+      <c r="B750" s="92"/>
     </row>
     <row r="751" ht="11.25" customHeight="1">
-      <c r="B751" s="95"/>
+      <c r="B751" s="92"/>
     </row>
     <row r="752" ht="11.25" customHeight="1">
-      <c r="B752" s="95"/>
+      <c r="B752" s="92"/>
     </row>
     <row r="753" ht="11.25" customHeight="1">
-      <c r="B753" s="95"/>
+      <c r="B753" s="92"/>
     </row>
     <row r="754" ht="11.25" customHeight="1">
-      <c r="B754" s="95"/>
+      <c r="B754" s="92"/>
     </row>
     <row r="755" ht="11.25" customHeight="1">
-      <c r="B755" s="95"/>
+      <c r="B755" s="92"/>
     </row>
     <row r="756" ht="11.25" customHeight="1">
-      <c r="B756" s="95"/>
+      <c r="B756" s="92"/>
     </row>
     <row r="757" ht="11.25" customHeight="1">
-      <c r="B757" s="95"/>
+      <c r="B757" s="92"/>
     </row>
     <row r="758" ht="11.25" customHeight="1">
-      <c r="B758" s="95"/>
+      <c r="B758" s="92"/>
     </row>
     <row r="759" ht="11.25" customHeight="1">
-      <c r="B759" s="95"/>
+      <c r="B759" s="92"/>
     </row>
     <row r="760" ht="11.25" customHeight="1">
-      <c r="B760" s="95"/>
+      <c r="B760" s="92"/>
     </row>
     <row r="761" ht="11.25" customHeight="1">
-      <c r="B761" s="95"/>
+      <c r="B761" s="92"/>
     </row>
     <row r="762" ht="11.25" customHeight="1">
-      <c r="B762" s="95"/>
+      <c r="B762" s="92"/>
     </row>
     <row r="763" ht="11.25" customHeight="1">
-      <c r="B763" s="95"/>
+      <c r="B763" s="92"/>
     </row>
     <row r="764" ht="11.25" customHeight="1">
-      <c r="B764" s="95"/>
+      <c r="B764" s="92"/>
     </row>
     <row r="765" ht="11.25" customHeight="1">
-      <c r="B765" s="95"/>
+      <c r="B765" s="92"/>
     </row>
     <row r="766" ht="11.25" customHeight="1">
-      <c r="B766" s="95"/>
+      <c r="B766" s="92"/>
     </row>
     <row r="767" ht="11.25" customHeight="1">
-      <c r="B767" s="95"/>
+      <c r="B767" s="92"/>
     </row>
     <row r="768" ht="11.25" customHeight="1">
-      <c r="B768" s="95"/>
+      <c r="B768" s="92"/>
     </row>
     <row r="769" ht="11.25" customHeight="1">
-      <c r="B769" s="95"/>
+      <c r="B769" s="92"/>
     </row>
     <row r="770" ht="11.25" customHeight="1">
-      <c r="B770" s="95"/>
+      <c r="B770" s="92"/>
     </row>
     <row r="771" ht="11.25" customHeight="1">
-      <c r="B771" s="95"/>
+      <c r="B771" s="92"/>
     </row>
     <row r="772" ht="11.25" customHeight="1">
-      <c r="B772" s="95"/>
+      <c r="B772" s="92"/>
     </row>
     <row r="773" ht="11.25" customHeight="1">
-      <c r="B773" s="95"/>
+      <c r="B773" s="92"/>
     </row>
     <row r="774" ht="11.25" customHeight="1">
-      <c r="B774" s="95"/>
+      <c r="B774" s="92"/>
     </row>
     <row r="775" ht="11.25" customHeight="1">
-      <c r="B775" s="95"/>
+      <c r="B775" s="92"/>
     </row>
     <row r="776" ht="11.25" customHeight="1">
-      <c r="B776" s="95"/>
+      <c r="B776" s="92"/>
     </row>
     <row r="777" ht="11.25" customHeight="1">
-      <c r="B777" s="95"/>
+      <c r="B777" s="92"/>
     </row>
     <row r="778" ht="11.25" customHeight="1">
-      <c r="B778" s="95"/>
+      <c r="B778" s="92"/>
     </row>
     <row r="779" ht="11.25" customHeight="1">
-      <c r="B779" s="95"/>
+      <c r="B779" s="92"/>
     </row>
     <row r="780" ht="11.25" customHeight="1">
-      <c r="B780" s="95"/>
+      <c r="B780" s="92"/>
     </row>
     <row r="781" ht="11.25" customHeight="1">
-      <c r="B781" s="95"/>
+      <c r="B781" s="92"/>
     </row>
     <row r="782" ht="11.25" customHeight="1">
-      <c r="B782" s="95"/>
+      <c r="B782" s="92"/>
     </row>
     <row r="783" ht="11.25" customHeight="1">
-      <c r="B783" s="95"/>
+      <c r="B783" s="92"/>
     </row>
     <row r="784" ht="11.25" customHeight="1">
-      <c r="B784" s="95"/>
+      <c r="B784" s="92"/>
     </row>
     <row r="785" ht="11.25" customHeight="1">
-      <c r="B785" s="95"/>
+      <c r="B785" s="92"/>
     </row>
     <row r="786" ht="11.25" customHeight="1">
-      <c r="B786" s="95"/>
+      <c r="B786" s="92"/>
     </row>
     <row r="787" ht="11.25" customHeight="1">
-      <c r="B787" s="95"/>
+      <c r="B787" s="92"/>
     </row>
     <row r="788" ht="11.25" customHeight="1">
-      <c r="B788" s="95"/>
+      <c r="B788" s="92"/>
     </row>
     <row r="789" ht="11.25" customHeight="1">
-      <c r="B789" s="95"/>
+      <c r="B789" s="92"/>
     </row>
     <row r="790" ht="11.25" customHeight="1">
-      <c r="B790" s="95"/>
+      <c r="B790" s="92"/>
     </row>
     <row r="791" ht="11.25" customHeight="1">
-      <c r="B791" s="95"/>
+      <c r="B791" s="92"/>
     </row>
     <row r="792" ht="11.25" customHeight="1">
-      <c r="B792" s="95"/>
+      <c r="B792" s="92"/>
     </row>
     <row r="793" ht="11.25" customHeight="1">
-      <c r="B793" s="95"/>
+      <c r="B793" s="92"/>
     </row>
     <row r="794" ht="11.25" customHeight="1">
-      <c r="B794" s="95"/>
+      <c r="B794" s="92"/>
     </row>
     <row r="795" ht="11.25" customHeight="1">
-      <c r="B795" s="95"/>
+      <c r="B795" s="92"/>
     </row>
     <row r="796" ht="11.25" customHeight="1">
-      <c r="B796" s="95"/>
+      <c r="B796" s="92"/>
     </row>
     <row r="797" ht="11.25" customHeight="1">
-      <c r="B797" s="95"/>
+      <c r="B797" s="92"/>
     </row>
     <row r="798" ht="11.25" customHeight="1">
-      <c r="B798" s="95"/>
+      <c r="B798" s="92"/>
     </row>
     <row r="799" ht="11.25" customHeight="1">
-      <c r="B799" s="95"/>
+      <c r="B799" s="92"/>
     </row>
     <row r="800" ht="11.25" customHeight="1">
-      <c r="B800" s="95"/>
+      <c r="B800" s="92"/>
     </row>
     <row r="801" ht="11.25" customHeight="1">
-      <c r="B801" s="95"/>
+      <c r="B801" s="92"/>
     </row>
     <row r="802" ht="11.25" customHeight="1">
-      <c r="B802" s="95"/>
+      <c r="B802" s="92"/>
     </row>
     <row r="803" ht="11.25" customHeight="1">
-      <c r="B803" s="95"/>
+      <c r="B803" s="92"/>
     </row>
     <row r="804" ht="11.25" customHeight="1">
-      <c r="B804" s="95"/>
+      <c r="B804" s="92"/>
     </row>
     <row r="805" ht="11.25" customHeight="1">
-      <c r="B805" s="95"/>
+      <c r="B805" s="92"/>
     </row>
     <row r="806" ht="11.25" customHeight="1">
-      <c r="B806" s="95"/>
+      <c r="B806" s="92"/>
     </row>
     <row r="807" ht="11.25" customHeight="1">
-      <c r="B807" s="95"/>
+      <c r="B807" s="92"/>
     </row>
     <row r="808" ht="11.25" customHeight="1">
-      <c r="B808" s="95"/>
+      <c r="B808" s="92"/>
     </row>
     <row r="809" ht="11.25" customHeight="1">
-      <c r="B809" s="95"/>
+      <c r="B809" s="92"/>
     </row>
     <row r="810" ht="11.25" customHeight="1">
-      <c r="B810" s="95"/>
+      <c r="B810" s="92"/>
     </row>
     <row r="811" ht="11.25" customHeight="1">
-      <c r="B811" s="95"/>
+      <c r="B811" s="92"/>
     </row>
     <row r="812" ht="11.25" customHeight="1">
-      <c r="B812" s="95"/>
+      <c r="B812" s="92"/>
     </row>
     <row r="813" ht="11.25" customHeight="1">
-      <c r="B813" s="95"/>
+      <c r="B813" s="92"/>
     </row>
     <row r="814" ht="11.25" customHeight="1">
-      <c r="B814" s="95"/>
+      <c r="B814" s="92"/>
     </row>
     <row r="815" ht="11.25" customHeight="1">
-      <c r="B815" s="95"/>
+      <c r="B815" s="92"/>
     </row>
     <row r="816" ht="11.25" customHeight="1">
-      <c r="B816" s="95"/>
+      <c r="B816" s="92"/>
     </row>
     <row r="817" ht="11.25" customHeight="1">
-      <c r="B817" s="95"/>
+      <c r="B817" s="92"/>
     </row>
     <row r="818" ht="11.25" customHeight="1">
-      <c r="B818" s="95"/>
+      <c r="B818" s="92"/>
     </row>
     <row r="819" ht="11.25" customHeight="1">
-      <c r="B819" s="95"/>
+      <c r="B819" s="92"/>
     </row>
     <row r="820" ht="11.25" customHeight="1">
-      <c r="B820" s="95"/>
+      <c r="B820" s="92"/>
     </row>
     <row r="821" ht="11.25" customHeight="1">
-      <c r="B821" s="95"/>
+      <c r="B821" s="92"/>
     </row>
     <row r="822" ht="11.25" customHeight="1">
-      <c r="B822" s="95"/>
+      <c r="B822" s="92"/>
     </row>
     <row r="823" ht="11.25" customHeight="1">
-      <c r="B823" s="95"/>
+      <c r="B823" s="92"/>
     </row>
     <row r="824" ht="11.25" customHeight="1">
-      <c r="B824" s="95"/>
+      <c r="B824" s="92"/>
     </row>
     <row r="825" ht="11.25" customHeight="1">
-      <c r="B825" s="95"/>
+      <c r="B825" s="92"/>
     </row>
     <row r="826" ht="11.25" customHeight="1">
-      <c r="B826" s="95"/>
+      <c r="B826" s="92"/>
     </row>
     <row r="827" ht="11.25" customHeight="1">
-      <c r="B827" s="95"/>
+      <c r="B827" s="92"/>
     </row>
     <row r="828" ht="11.25" customHeight="1">
-      <c r="B828" s="95"/>
+      <c r="B828" s="92"/>
     </row>
     <row r="829" ht="11.25" customHeight="1">
-      <c r="B829" s="95"/>
+      <c r="B829" s="92"/>
     </row>
     <row r="830" ht="11.25" customHeight="1">
-      <c r="B830" s="95"/>
+      <c r="B830" s="92"/>
     </row>
     <row r="831" ht="11.25" customHeight="1">
-      <c r="B831" s="95"/>
+      <c r="B831" s="92"/>
     </row>
     <row r="832" ht="11.25" customHeight="1">
-      <c r="B832" s="95"/>
+      <c r="B832" s="92"/>
     </row>
     <row r="833" ht="11.25" customHeight="1">
-      <c r="B833" s="95"/>
+      <c r="B833" s="92"/>
     </row>
     <row r="834" ht="11.25" customHeight="1">
-      <c r="B834" s="95"/>
+      <c r="B834" s="92"/>
     </row>
     <row r="835" ht="11.25" customHeight="1">
-      <c r="B835" s="95"/>
+      <c r="B835" s="92"/>
     </row>
     <row r="836" ht="11.25" customHeight="1">
-      <c r="B836" s="95"/>
+      <c r="B836" s="92"/>
     </row>
     <row r="837" ht="11.25" customHeight="1">
-      <c r="B837" s="95"/>
+      <c r="B837" s="92"/>
     </row>
     <row r="838" ht="11.25" customHeight="1">
-      <c r="B838" s="95"/>
+      <c r="B838" s="92"/>
     </row>
     <row r="839" ht="11.25" customHeight="1">
-      <c r="B839" s="95"/>
+      <c r="B839" s="92"/>
     </row>
     <row r="840" ht="11.25" customHeight="1">
-      <c r="B840" s="95"/>
+      <c r="B840" s="92"/>
     </row>
     <row r="841" ht="11.25" customHeight="1">
-      <c r="B841" s="95"/>
+      <c r="B841" s="92"/>
     </row>
     <row r="842" ht="11.25" customHeight="1">
-      <c r="B842" s="95"/>
+      <c r="B842" s="92"/>
     </row>
     <row r="843" ht="11.25" customHeight="1">
-      <c r="B843" s="95"/>
+      <c r="B843" s="92"/>
     </row>
     <row r="844" ht="11.25" customHeight="1">
-      <c r="B844" s="95"/>
+      <c r="B844" s="92"/>
     </row>
     <row r="845" ht="11.25" customHeight="1">
-      <c r="B845" s="95"/>
+      <c r="B845" s="92"/>
     </row>
     <row r="846" ht="11.25" customHeight="1">
-      <c r="B846" s="95"/>
+      <c r="B846" s="92"/>
     </row>
     <row r="847" ht="11.25" customHeight="1">
-      <c r="B847" s="95"/>
+      <c r="B847" s="92"/>
     </row>
     <row r="848" ht="11.25" customHeight="1">
-      <c r="B848" s="95"/>
+      <c r="B848" s="92"/>
     </row>
     <row r="849" ht="11.25" customHeight="1">
-      <c r="B849" s="95"/>
+      <c r="B849" s="92"/>
     </row>
     <row r="850" ht="11.25" customHeight="1">
-      <c r="B850" s="95"/>
+      <c r="B850" s="92"/>
     </row>
     <row r="851" ht="11.25" customHeight="1">
-      <c r="B851" s="95"/>
+      <c r="B851" s="92"/>
     </row>
     <row r="852" ht="11.25" customHeight="1">
-      <c r="B852" s="95"/>
+      <c r="B852" s="92"/>
     </row>
     <row r="853" ht="11.25" customHeight="1">
-      <c r="B853" s="95"/>
+      <c r="B853" s="92"/>
     </row>
     <row r="854" ht="11.25" customHeight="1">
-      <c r="B854" s="95"/>
+      <c r="B854" s="92"/>
     </row>
     <row r="855" ht="11.25" customHeight="1">
-      <c r="B855" s="95"/>
+      <c r="B855" s="92"/>
     </row>
     <row r="856" ht="11.25" customHeight="1">
-      <c r="B856" s="95"/>
+      <c r="B856" s="92"/>
     </row>
     <row r="857" ht="11.25" customHeight="1">
-      <c r="B857" s="95"/>
+      <c r="B857" s="92"/>
     </row>
     <row r="858" ht="11.25" customHeight="1">
-      <c r="B858" s="95"/>
+      <c r="B858" s="92"/>
     </row>
     <row r="859" ht="11.25" customHeight="1">
-      <c r="B859" s="95"/>
+      <c r="B859" s="92"/>
     </row>
     <row r="860" ht="11.25" customHeight="1">
-      <c r="B860" s="95"/>
+      <c r="B860" s="92"/>
     </row>
     <row r="861" ht="11.25" customHeight="1">
-      <c r="B861" s="95"/>
+      <c r="B861" s="92"/>
     </row>
     <row r="862" ht="11.25" customHeight="1">
-      <c r="B862" s="95"/>
+      <c r="B862" s="92"/>
     </row>
     <row r="863" ht="11.25" customHeight="1">
-      <c r="B863" s="95"/>
+      <c r="B863" s="92"/>
     </row>
     <row r="864" ht="11.25" customHeight="1">
-      <c r="B864" s="95"/>
+      <c r="B864" s="92"/>
     </row>
     <row r="865" ht="11.25" customHeight="1">
-      <c r="B865" s="95"/>
+      <c r="B865" s="92"/>
     </row>
     <row r="866" ht="11.25" customHeight="1">
-      <c r="B866" s="95"/>
+      <c r="B866" s="92"/>
     </row>
     <row r="867" ht="11.25" customHeight="1">
-      <c r="B867" s="95"/>
+      <c r="B867" s="92"/>
     </row>
     <row r="868" ht="11.25" customHeight="1">
-      <c r="B868" s="95"/>
+      <c r="B868" s="92"/>
     </row>
     <row r="869" ht="11.25" customHeight="1">
-      <c r="B869" s="95"/>
+      <c r="B869" s="92"/>
     </row>
     <row r="870" ht="11.25" customHeight="1">
-      <c r="B870" s="95"/>
+      <c r="B870" s="92"/>
     </row>
     <row r="871" ht="11.25" customHeight="1">
-      <c r="B871" s="95"/>
+      <c r="B871" s="92"/>
     </row>
     <row r="872" ht="11.25" customHeight="1">
-      <c r="B872" s="95"/>
+      <c r="B872" s="92"/>
     </row>
     <row r="873" ht="11.25" customHeight="1">
-      <c r="B873" s="95"/>
+      <c r="B873" s="92"/>
     </row>
     <row r="874" ht="11.25" customHeight="1">
-      <c r="B874" s="95"/>
+      <c r="B874" s="92"/>
     </row>
     <row r="875" ht="11.25" customHeight="1">
-      <c r="B875" s="95"/>
+      <c r="B875" s="92"/>
     </row>
     <row r="876" ht="11.25" customHeight="1">
-      <c r="B876" s="95"/>
+      <c r="B876" s="92"/>
     </row>
     <row r="877" ht="11.25" customHeight="1">
-      <c r="B877" s="95"/>
+      <c r="B877" s="92"/>
     </row>
     <row r="878" ht="11.25" customHeight="1">
-      <c r="B878" s="95"/>
+      <c r="B878" s="92"/>
     </row>
     <row r="879" ht="11.25" customHeight="1">
-      <c r="B879" s="95"/>
+      <c r="B879" s="92"/>
     </row>
     <row r="880" ht="11.25" customHeight="1">
-      <c r="B880" s="95"/>
+      <c r="B880" s="92"/>
     </row>
     <row r="881" ht="11.25" customHeight="1">
-      <c r="B881" s="95"/>
+      <c r="B881" s="92"/>
     </row>
     <row r="882" ht="11.25" customHeight="1">
-      <c r="B882" s="95"/>
+      <c r="B882" s="92"/>
     </row>
     <row r="883" ht="11.25" customHeight="1">
-      <c r="B883" s="95"/>
+      <c r="B883" s="92"/>
     </row>
     <row r="884" ht="11.25" customHeight="1">
-      <c r="B884" s="95"/>
+      <c r="B884" s="92"/>
     </row>
     <row r="885" ht="11.25" customHeight="1">
-      <c r="B885" s="95"/>
+      <c r="B885" s="92"/>
     </row>
     <row r="886" ht="11.25" customHeight="1">
-      <c r="B886" s="95"/>
+      <c r="B886" s="92"/>
     </row>
     <row r="887" ht="11.25" customHeight="1">
-      <c r="B887" s="95"/>
+      <c r="B887" s="92"/>
     </row>
     <row r="888" ht="11.25" customHeight="1">
-      <c r="B888" s="95"/>
+      <c r="B888" s="92"/>
     </row>
     <row r="889" ht="11.25" customHeight="1">
-      <c r="B889" s="95"/>
+      <c r="B889" s="92"/>
     </row>
     <row r="890" ht="11.25" customHeight="1">
-      <c r="B890" s="95"/>
+      <c r="B890" s="92"/>
     </row>
     <row r="891" ht="11.25" customHeight="1">
-      <c r="B891" s="95"/>
+      <c r="B891" s="92"/>
     </row>
     <row r="892" ht="11.25" customHeight="1">
-      <c r="B892" s="95"/>
+      <c r="B892" s="92"/>
     </row>
     <row r="893" ht="11.25" customHeight="1">
-      <c r="B893" s="95"/>
+      <c r="B893" s="92"/>
     </row>
     <row r="894" ht="11.25" customHeight="1">
-      <c r="B894" s="95"/>
+      <c r="B894" s="92"/>
     </row>
     <row r="895" ht="11.25" customHeight="1">
-      <c r="B895" s="95"/>
+      <c r="B895" s="92"/>
     </row>
     <row r="896" ht="11.25" customHeight="1">
-      <c r="B896" s="95"/>
+      <c r="B896" s="92"/>
     </row>
     <row r="897" ht="11.25" customHeight="1">
-      <c r="B897" s="95"/>
+      <c r="B897" s="92"/>
     </row>
     <row r="898" ht="11.25" customHeight="1">
-      <c r="B898" s="95"/>
+      <c r="B898" s="92"/>
     </row>
     <row r="899" ht="11.25" customHeight="1">
-      <c r="B899" s="95"/>
+      <c r="B899" s="92"/>
     </row>
     <row r="900" ht="11.25" customHeight="1">
-      <c r="B900" s="95"/>
+      <c r="B900" s="92"/>
     </row>
     <row r="901" ht="11.25" customHeight="1">
-      <c r="B901" s="95"/>
+      <c r="B901" s="92"/>
     </row>
     <row r="902" ht="11.25" customHeight="1">
-      <c r="B902" s="95"/>
+      <c r="B902" s="92"/>
     </row>
     <row r="903" ht="11.25" customHeight="1">
-      <c r="B903" s="95"/>
+      <c r="B903" s="92"/>
     </row>
     <row r="904" ht="11.25" customHeight="1">
-      <c r="B904" s="95"/>
+      <c r="B904" s="92"/>
     </row>
     <row r="905" ht="11.25" customHeight="1">
-      <c r="B905" s="95"/>
+      <c r="B905" s="92"/>
     </row>
     <row r="906" ht="11.25" customHeight="1">
-      <c r="B906" s="95"/>
+      <c r="B906" s="92"/>
     </row>
     <row r="907" ht="11.25" customHeight="1">
-      <c r="B907" s="95"/>
+      <c r="B907" s="92"/>
     </row>
     <row r="908" ht="11.25" customHeight="1">
-      <c r="B908" s="95"/>
+      <c r="B908" s="92"/>
     </row>
     <row r="909" ht="11.25" customHeight="1">
-      <c r="B909" s="95"/>
+      <c r="B909" s="92"/>
     </row>
     <row r="910" ht="11.25" customHeight="1">
-      <c r="B910" s="95"/>
+      <c r="B910" s="92"/>
     </row>
     <row r="911" ht="11.25" customHeight="1">
-      <c r="B911" s="95"/>
+      <c r="B911" s="92"/>
     </row>
     <row r="912" ht="11.25" customHeight="1">
-      <c r="B912" s="95"/>
+      <c r="B912" s="92"/>
     </row>
     <row r="913" ht="11.25" customHeight="1">
-      <c r="B913" s="95"/>
+      <c r="B913" s="92"/>
     </row>
     <row r="914" ht="11.25" customHeight="1">
-      <c r="B914" s="95"/>
+      <c r="B914" s="92"/>
     </row>
     <row r="915" ht="11.25" customHeight="1">
-      <c r="B915" s="95"/>
+      <c r="B915" s="92"/>
     </row>
     <row r="916" ht="11.25" customHeight="1">
-      <c r="B916" s="95"/>
+      <c r="B916" s="92"/>
     </row>
     <row r="917" ht="11.25" customHeight="1">
-      <c r="B917" s="95"/>
+      <c r="B917" s="92"/>
     </row>
     <row r="918" ht="11.25" customHeight="1">
-      <c r="B918" s="95"/>
+      <c r="B918" s="92"/>
     </row>
     <row r="919" ht="11.25" customHeight="1">
-      <c r="B919" s="95"/>
+      <c r="B919" s="92"/>
     </row>
     <row r="920" ht="11.25" customHeight="1">
-      <c r="B920" s="95"/>
+      <c r="B920" s="92"/>
     </row>
     <row r="921" ht="11.25" customHeight="1">
-      <c r="B921" s="95"/>
+      <c r="B921" s="92"/>
     </row>
     <row r="922" ht="11.25" customHeight="1">
-      <c r="B922" s="95"/>
+      <c r="B922" s="92"/>
     </row>
     <row r="923" ht="11.25" customHeight="1">
-      <c r="B923" s="95"/>
+      <c r="B923" s="92"/>
     </row>
     <row r="924" ht="11.25" customHeight="1">
-      <c r="B924" s="95"/>
+      <c r="B924" s="92"/>
     </row>
     <row r="925" ht="11.25" customHeight="1">
-      <c r="B925" s="95"/>
+      <c r="B925" s="92"/>
     </row>
     <row r="926" ht="11.25" customHeight="1">
-      <c r="B926" s="95"/>
+      <c r="B926" s="92"/>
     </row>
     <row r="927" ht="11.25" customHeight="1">
-      <c r="B927" s="95"/>
+      <c r="B927" s="92"/>
     </row>
     <row r="928" ht="11.25" customHeight="1">
-      <c r="B928" s="95"/>
+      <c r="B928" s="92"/>
     </row>
     <row r="929" ht="11.25" customHeight="1">
-      <c r="B929" s="95"/>
+      <c r="B929" s="92"/>
     </row>
     <row r="930" ht="11.25" customHeight="1">
-      <c r="B930" s="95"/>
+      <c r="B930" s="92"/>
     </row>
     <row r="931" ht="11.25" customHeight="1">
-      <c r="B931" s="95"/>
+      <c r="B931" s="92"/>
     </row>
     <row r="932" ht="11.25" customHeight="1">
-      <c r="B932" s="95"/>
+      <c r="B932" s="92"/>
     </row>
     <row r="933" ht="11.25" customHeight="1">
-      <c r="B933" s="95"/>
+      <c r="B933" s="92"/>
     </row>
     <row r="934" ht="11.25" customHeight="1">
-      <c r="B934" s="95"/>
+      <c r="B934" s="92"/>
     </row>
     <row r="935" ht="11.25" customHeight="1">
-      <c r="B935" s="95"/>
+      <c r="B935" s="92"/>
     </row>
     <row r="936" ht="11.25" customHeight="1">
-      <c r="B936" s="95"/>
+      <c r="B936" s="92"/>
     </row>
     <row r="937" ht="11.25" customHeight="1">
-      <c r="B937" s="95"/>
+      <c r="B937" s="92"/>
     </row>
     <row r="938" ht="11.25" customHeight="1">
-      <c r="B938" s="95"/>
+      <c r="B938" s="92"/>
     </row>
     <row r="939" ht="11.25" customHeight="1">
-      <c r="B939" s="95"/>
+      <c r="B939" s="92"/>
     </row>
     <row r="940" ht="11.25" customHeight="1">
-      <c r="B940" s="95"/>
+      <c r="B940" s="92"/>
     </row>
     <row r="941" ht="11.25" customHeight="1">
-      <c r="B941" s="95"/>
+      <c r="B941" s="92"/>
     </row>
     <row r="942" ht="11.25" customHeight="1">
-      <c r="B942" s="95"/>
+      <c r="B942" s="92"/>
     </row>
     <row r="943" ht="11.25" customHeight="1">
-      <c r="B943" s="95"/>
+      <c r="B943" s="92"/>
     </row>
     <row r="944" ht="11.25" customHeight="1">
-      <c r="B944" s="95"/>
+      <c r="B944" s="92"/>
     </row>
     <row r="945" ht="11.25" customHeight="1">
-      <c r="B945" s="95"/>
+      <c r="B945" s="92"/>
     </row>
     <row r="946" ht="11.25" customHeight="1">
-      <c r="B946" s="95"/>
+      <c r="B946" s="92"/>
     </row>
     <row r="947" ht="11.25" customHeight="1">
-      <c r="B947" s="95"/>
+      <c r="B947" s="92"/>
     </row>
     <row r="948" ht="11.25" customHeight="1">
-      <c r="B948" s="95"/>
+      <c r="B948" s="92"/>
     </row>
     <row r="949" ht="11.25" customHeight="1">
-      <c r="B949" s="95"/>
+      <c r="B949" s="92"/>
     </row>
     <row r="950" ht="11.25" customHeight="1">
-      <c r="B950" s="95"/>
+      <c r="B950" s="92"/>
     </row>
     <row r="951" ht="11.25" customHeight="1">
-      <c r="B951" s="95"/>
+      <c r="B951" s="92"/>
     </row>
     <row r="952" ht="11.25" customHeight="1">
-      <c r="B952" s="95"/>
+      <c r="B952" s="92"/>
     </row>
     <row r="953" ht="11.25" customHeight="1">
-      <c r="B953" s="95"/>
+      <c r="B953" s="92"/>
     </row>
     <row r="954" ht="11.25" customHeight="1">
-      <c r="B954" s="95"/>
+      <c r="B954" s="92"/>
     </row>
     <row r="955" ht="11.25" customHeight="1">
-      <c r="B955" s="95"/>
+      <c r="B955" s="92"/>
     </row>
     <row r="956" ht="11.25" customHeight="1">
-      <c r="B956" s="95"/>
+      <c r="B956" s="92"/>
     </row>
     <row r="957" ht="11.25" customHeight="1">
-      <c r="B957" s="95"/>
+      <c r="B957" s="92"/>
     </row>
     <row r="958" ht="11.25" customHeight="1">
-      <c r="B958" s="95"/>
+      <c r="B958" s="92"/>
     </row>
     <row r="959" ht="11.25" customHeight="1">
-      <c r="B959" s="95"/>
+      <c r="B959" s="92"/>
     </row>
     <row r="960" ht="11.25" customHeight="1">
-      <c r="B960" s="95"/>
+      <c r="B960" s="92"/>
     </row>
     <row r="961" ht="11.25" customHeight="1">
-      <c r="B961" s="95"/>
+      <c r="B961" s="92"/>
     </row>
     <row r="962" ht="11.25" customHeight="1">
-      <c r="B962" s="95"/>
+      <c r="B962" s="92"/>
     </row>
     <row r="963" ht="11.25" customHeight="1">
-      <c r="B963" s="95"/>
+      <c r="B963" s="92"/>
     </row>
     <row r="964" ht="11.25" customHeight="1">
-      <c r="B964" s="95"/>
+      <c r="B964" s="92"/>
     </row>
     <row r="965" ht="11.25" customHeight="1">
-      <c r="B965" s="95"/>
+      <c r="B965" s="92"/>
     </row>
     <row r="966" ht="11.25" customHeight="1">
-      <c r="B966" s="95"/>
+      <c r="B966" s="92"/>
     </row>
     <row r="967" ht="11.25" customHeight="1">
-      <c r="B967" s="95"/>
+      <c r="B967" s="92"/>
     </row>
     <row r="968" ht="11.25" customHeight="1">
-      <c r="B968" s="95"/>
+      <c r="B968" s="92"/>
     </row>
     <row r="969" ht="11.25" customHeight="1">
-      <c r="B969" s="95"/>
+      <c r="B969" s="92"/>
     </row>
     <row r="970" ht="11.25" customHeight="1">
-      <c r="B970" s="95"/>
+      <c r="B970" s="92"/>
     </row>
     <row r="971" ht="11.25" customHeight="1">
-      <c r="B971" s="95"/>
+      <c r="B971" s="92"/>
     </row>
     <row r="972" ht="11.25" customHeight="1">
-      <c r="B972" s="95"/>
+      <c r="B972" s="92"/>
     </row>
     <row r="973" ht="11.25" customHeight="1">
-      <c r="B973" s="95"/>
+      <c r="B973" s="92"/>
     </row>
     <row r="974" ht="11.25" customHeight="1">
-      <c r="B974" s="95"/>
+      <c r="B974" s="92"/>
     </row>
     <row r="975" ht="11.25" customHeight="1">
-      <c r="B975" s="95"/>
+      <c r="B975" s="92"/>
     </row>
     <row r="976" ht="11.25" customHeight="1">
-      <c r="B976" s="95"/>
+      <c r="B976" s="92"/>
     </row>
     <row r="977" ht="11.25" customHeight="1">
-      <c r="B977" s="95"/>
+      <c r="B977" s="92"/>
     </row>
     <row r="978" ht="11.25" customHeight="1">
-      <c r="B978" s="95"/>
+      <c r="B978" s="92"/>
     </row>
     <row r="979" ht="11.25" customHeight="1">
-      <c r="B979" s="95"/>
+      <c r="B979" s="92"/>
     </row>
     <row r="980" ht="11.25" customHeight="1">
-      <c r="B980" s="95"/>
+      <c r="B980" s="92"/>
     </row>
     <row r="981" ht="11.25" customHeight="1">
-      <c r="B981" s="95"/>
+      <c r="B981" s="92"/>
     </row>
     <row r="982" ht="11.25" customHeight="1">
-      <c r="B982" s="95"/>
+      <c r="B982" s="92"/>
     </row>
     <row r="983" ht="11.25" customHeight="1">
-      <c r="B983" s="95"/>
+      <c r="B983" s="92"/>
     </row>
     <row r="984" ht="11.25" customHeight="1">
-      <c r="B984" s="95"/>
+      <c r="B984" s="92"/>
     </row>
     <row r="985" ht="11.25" customHeight="1">
-      <c r="B985" s="95"/>
+      <c r="B985" s="92"/>
     </row>
     <row r="986" ht="11.25" customHeight="1">
-      <c r="B986" s="95"/>
+      <c r="B986" s="92"/>
     </row>
     <row r="987" ht="11.25" customHeight="1">
-      <c r="B987" s="95"/>
+      <c r="B987" s="92"/>
     </row>
     <row r="988" ht="11.25" customHeight="1">
-      <c r="B988" s="95"/>
+      <c r="B988" s="92"/>
     </row>
     <row r="989" ht="11.25" customHeight="1">
-      <c r="B989" s="95"/>
+      <c r="B989" s="92"/>
     </row>
     <row r="990" ht="11.25" customHeight="1">
-      <c r="B990" s="95"/>
+      <c r="B990" s="92"/>
     </row>
     <row r="991" ht="11.25" customHeight="1">
-      <c r="B991" s="95"/>
+      <c r="B991" s="92"/>
     </row>
     <row r="992" ht="11.25" customHeight="1">
-      <c r="B992" s="95"/>
+      <c r="B992" s="92"/>
     </row>
     <row r="993" ht="11.25" customHeight="1">
-      <c r="B993" s="95"/>
+      <c r="B993" s="92"/>
     </row>
     <row r="994" ht="11.25" customHeight="1">
-      <c r="B994" s="95"/>
+      <c r="B994" s="92"/>
     </row>
     <row r="995" ht="11.25" customHeight="1">
-      <c r="B995" s="95"/>
+      <c r="B995" s="92"/>
     </row>
     <row r="996" ht="11.25" customHeight="1">
-      <c r="B996" s="95"/>
+      <c r="B996" s="92"/>
     </row>
     <row r="997" ht="11.25" customHeight="1">
-      <c r="B997" s="95"/>
+      <c r="B997" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="20">

</xml_diff>